<commit_message>
nn and minutes to models
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -4,16 +4,16 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="24030"/>
   <workbookPr showInkAnnotation="0" hidePivotFieldList="1" autoCompressPictures="0"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="15540" tabRatio="500" activeTab="1"/>
+    <workbookView xWindow="1120" yWindow="1120" windowWidth="24480" windowHeight="14420" tabRatio="500" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet5" sheetId="5" r:id="rId2"/>
     <sheet name="Sheet4" sheetId="4" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="140000" calcMode="manual" concurrentCalc="0"/>
+  <calcPr calcId="140000" concurrentCalc="0"/>
   <pivotCaches>
-    <pivotCache cacheId="12" r:id="rId4"/>
+    <pivotCache cacheId="3" r:id="rId4"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{7523E5D3-25F3-A5E0-1632-64F254C22452}">
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="73">
   <si>
     <t>Date</t>
   </si>
@@ -145,6 +145,105 @@
   <si>
     <t>S130000006</t>
   </si>
+  <si>
+    <t>S130611118</t>
+  </si>
+  <si>
+    <t>S130611542</t>
+  </si>
+  <si>
+    <t>S130611988</t>
+  </si>
+  <si>
+    <t>S130612327</t>
+  </si>
+  <si>
+    <t>S130612801</t>
+  </si>
+  <si>
+    <t>S131244958</t>
+  </si>
+  <si>
+    <t>S131245950</t>
+  </si>
+  <si>
+    <t>S132293712</t>
+  </si>
+  <si>
+    <t>S132294089</t>
+  </si>
+  <si>
+    <t>S132533642</t>
+  </si>
+  <si>
+    <t>S132535745</t>
+  </si>
+  <si>
+    <t>S132537184</t>
+  </si>
+  <si>
+    <t>S133093188</t>
+  </si>
+  <si>
+    <t>S133094607</t>
+  </si>
+  <si>
+    <t>S133095435</t>
+  </si>
+  <si>
+    <t>S133097181</t>
+  </si>
+  <si>
+    <t>NN</t>
+  </si>
+  <si>
+    <t>S133641750</t>
+  </si>
+  <si>
+    <t>S133642428</t>
+  </si>
+  <si>
+    <t>S133642781</t>
+  </si>
+  <si>
+    <t>S133643274</t>
+  </si>
+  <si>
+    <t>S134270174</t>
+  </si>
+  <si>
+    <t>S134269016</t>
+  </si>
+  <si>
+    <t>S134269582</t>
+  </si>
+  <si>
+    <t>S134271406</t>
+  </si>
+  <si>
+    <t>S134271964</t>
+  </si>
+  <si>
+    <t>S135020132</t>
+  </si>
+  <si>
+    <t>S135020740</t>
+  </si>
+  <si>
+    <t>S135023095</t>
+  </si>
+  <si>
+    <t>S135023734</t>
+  </si>
+  <si>
+    <t>S135326936</t>
+  </si>
+  <si>
+    <t>S135327115</t>
+  </si>
+  <si>
+    <t>S135327370</t>
+  </si>
 </sst>
 </file>
 
@@ -156,6 +255,7 @@
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <charset val="128"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -254,7 +354,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="115">
+  <cellStyleXfs count="162">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
@@ -337,6 +437,53 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
@@ -401,7 +548,7 @@
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="115">
+  <cellStyles count="162">
     <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="4" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="6" builtinId="9" hidden="1"/>
@@ -459,6 +606,30 @@
     <cellStyle name="Followed Hyperlink" xfId="110" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="112" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="114" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="116" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="118" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="120" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="122" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="124" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="126" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="128" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="129" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="131" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="133" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="135" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="137" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="139" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="141" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="143" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="145" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="147" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="149" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="151" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="153" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="155" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="157" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="159" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="161" builtinId="9" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="3" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="5" builtinId="8" hidden="1"/>
@@ -516,6 +687,29 @@
     <cellStyle name="Hyperlink" xfId="109" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="111" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="113" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="115" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="117" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="119" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="121" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="123" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="125" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="127" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="130" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="132" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="134" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="136" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="138" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="140" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="142" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="144" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="146" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="148" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="150" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="152" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="154" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="156" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="158" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="160" builtinId="8" hidden="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -550,10 +744,10 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet5!$A$5:$A$18</c:f>
+              <c:f>Sheet5!$A$5:$A$19</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="14"/>
+                <c:ptCount val="15"/>
                 <c:pt idx="0">
                   <c:v>150.0</c:v>
                 </c:pt>
@@ -596,56 +790,62 @@
                 <c:pt idx="13">
                   <c:v>280.0</c:v>
                 </c:pt>
+                <c:pt idx="14">
+                  <c:v>290.0</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet5!$B$5:$B$18</c:f>
+              <c:f>Sheet5!$B$5:$B$19</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="14"/>
+                <c:ptCount val="15"/>
                 <c:pt idx="0">
                   <c:v>1.0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2.0</c:v>
+                  <c:v>5.0</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>9.0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5.0</c:v>
+                  <c:v>6.0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>15.0</c:v>
+                  <c:v>19.0</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>2.0</c:v>
+                  <c:v>6.0</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>18.0</c:v>
+                  <c:v>28.0</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>9.0</c:v>
+                  <c:v>20.0</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>9.0</c:v>
+                  <c:v>13.0</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>7.0</c:v>
+                  <c:v>11.0</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>13.0</c:v>
+                  <c:v>14.0</c:v>
                 </c:pt>
                 <c:pt idx="11">
                   <c:v>3.0</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>5.0</c:v>
+                  <c:v>9.0</c:v>
                 </c:pt>
                 <c:pt idx="13">
                   <c:v>2.0</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>1.0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -660,8 +860,8 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="150"/>
-        <c:axId val="-2090754408"/>
-        <c:axId val="-2133061752"/>
+        <c:axId val="-2125646632"/>
+        <c:axId val="-2125738872"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -674,10 +874,10 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet5!$V$3:$V$16</c:f>
+              <c:f>Sheet5!$V$3:$V$17</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="14"/>
+                <c:ptCount val="15"/>
                 <c:pt idx="0">
                   <c:v>150.0</c:v>
                 </c:pt>
@@ -720,56 +920,62 @@
                 <c:pt idx="13">
                   <c:v>280.0</c:v>
                 </c:pt>
+                <c:pt idx="14">
+                  <c:v>290.0</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet5!$W$3:$W$16</c:f>
+              <c:f>Sheet5!$W$3:$W$17</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="14"/>
+                <c:ptCount val="15"/>
                 <c:pt idx="0">
-                  <c:v>0.00131912664842662</c:v>
+                  <c:v>0.00113936331686994</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.00248593068935784</c:v>
+                  <c:v>0.00223901419611758</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.00422517514181524</c:v>
+                  <c:v>0.00394603925093226</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.00647669721644443</c:v>
+                  <c:v>0.00623700214952315</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.00895397033022763</c:v>
+                  <c:v>0.00884097832545786</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.0111642842596271</c:v>
+                  <c:v>0.0112391818255554</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.0125544964647117</c:v>
+                  <c:v>0.012813831471045</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.0127327112372427</c:v>
+                  <c:v>0.0131018691457743</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.0116465061212589</c:v>
+                  <c:v>0.012014271630392</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.00960779231948683</c:v>
+                  <c:v>0.00988033283984121</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.00714833229264748</c:v>
+                  <c:v>0.00728711532168424</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.00479666111541324</c:v>
+                  <c:v>0.00482002897793604</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.00290286285891706</c:v>
+                  <c:v>0.00285925964781033</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>0.00158440855658821</c:v>
+                  <c:v>0.00152113402352969</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.00072575711948566</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -786,11 +992,11 @@
         </c:dLbls>
         <c:marker val="1"/>
         <c:smooth val="0"/>
-        <c:axId val="-2090080968"/>
-        <c:axId val="-2090397352"/>
+        <c:axId val="-2125732408"/>
+        <c:axId val="-2125741912"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="-2090080968"/>
+        <c:axId val="-2125732408"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -800,7 +1006,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="-2090397352"/>
+        <c:crossAx val="-2125741912"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -808,7 +1014,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="-2090397352"/>
+        <c:axId val="-2125741912"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -819,12 +1025,12 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="-2090080968"/>
+        <c:crossAx val="-2125732408"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="-2133061752"/>
+        <c:axId val="-2125738872"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -834,12 +1040,12 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="-2090754408"/>
+        <c:crossAx val="-2125646632"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:catAx>
-        <c:axId val="-2090754408"/>
+        <c:axId val="-2125646632"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -849,7 +1055,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="-2133061752"/>
+        <c:crossAx val="-2125738872"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -910,16 +1116,16 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1" refreshedBy="Jesse Green" refreshedDate="42038.406953587961" createdVersion="4" refreshedVersion="4" minRefreshableVersion="3" recordCount="100">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1" refreshedBy="Jesse Green" refreshedDate="42047.398584490744" createdVersion="4" refreshedVersion="4" minRefreshableVersion="3" recordCount="147">
   <cacheSource type="worksheet">
-    <worksheetSource ref="A1:F101" sheet="Sheet4"/>
+    <worksheetSource ref="A1:F148" sheet="Sheet4"/>
   </cacheSource>
   <cacheFields count="6">
     <cacheField name="date" numFmtId="14">
-      <sharedItems containsSemiMixedTypes="0" containsNonDate="0" containsDate="1" containsString="0" minDate="2014-01-25T00:00:00" maxDate="2015-02-03T00:00:00"/>
+      <sharedItems containsSemiMixedTypes="0" containsNonDate="0" containsDate="1" containsString="0" minDate="2014-01-25T00:00:00" maxDate="2015-02-12T00:00:00"/>
     </cacheField>
     <cacheField name="score" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="152.30000000000001" maxValue="281.3"/>
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="152.30000000000001" maxValue="291.10000000000002"/>
     </cacheField>
     <cacheField name="model" numFmtId="0">
       <sharedItems/>
@@ -931,7 +1137,7 @@
       <sharedItems/>
     </cacheField>
     <cacheField name="rounded" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="150" maxValue="280" count="14">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="150" maxValue="290" count="15">
         <n v="240"/>
         <n v="170"/>
         <n v="220"/>
@@ -946,6 +1152,7 @@
         <n v="270"/>
         <n v="200"/>
         <n v="150"/>
+        <n v="290"/>
       </sharedItems>
     </cacheField>
   </cacheFields>
@@ -958,7 +1165,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" count="100">
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" count="147">
   <r>
     <d v="2015-01-15T00:00:00"/>
     <n v="235.4"/>
@@ -1758,13 +1965,389 @@
     <n v="8"/>
     <s v="l1"/>
     <x v="0"/>
+  </r>
+  <r>
+    <d v="2015-02-03T00:00:00"/>
+    <n v="272.2"/>
+    <s v="EN"/>
+    <n v="0"/>
+    <s v="l2"/>
+    <x v="11"/>
+  </r>
+  <r>
+    <d v="2015-02-03T00:00:00"/>
+    <n v="272.2"/>
+    <s v="EN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="11"/>
+  </r>
+  <r>
+    <d v="2015-02-03T00:00:00"/>
+    <n v="272.2"/>
+    <s v="EN"/>
+    <n v="0"/>
+    <s v="l1"/>
+    <x v="11"/>
+  </r>
+  <r>
+    <d v="2015-02-03T00:00:00"/>
+    <n v="272.2"/>
+    <s v="EN"/>
+    <n v="8"/>
+    <s v="l1"/>
+    <x v="11"/>
+  </r>
+  <r>
+    <d v="2015-02-03T00:00:00"/>
+    <n v="291.10000000000002"/>
+    <s v="SVR"/>
+    <n v="8"/>
+    <s v="l1"/>
+    <x v="14"/>
+  </r>
+  <r>
+    <d v="2015-02-04T00:00:00"/>
+    <n v="213"/>
+    <s v="EN"/>
+    <n v="0"/>
+    <s v="l2"/>
+    <x v="3"/>
+  </r>
+  <r>
+    <d v="2015-02-04T00:00:00"/>
+    <n v="229.7"/>
+    <s v="EN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="5"/>
+  </r>
+  <r>
+    <d v="2015-02-04T00:00:00"/>
+    <n v="199.2"/>
+    <s v="EN"/>
+    <n v="0"/>
+    <s v="l1"/>
+    <x v="12"/>
+  </r>
+  <r>
+    <d v="2015-02-04T00:00:00"/>
+    <n v="210.5"/>
+    <s v="EN"/>
+    <n v="8"/>
+    <s v="l1"/>
+    <x v="3"/>
+  </r>
+  <r>
+    <d v="2015-02-04T00:00:00"/>
+    <n v="218"/>
+    <s v="SVR"/>
+    <n v="8"/>
+    <s v="l1"/>
+    <x v="2"/>
+  </r>
+  <r>
+    <d v="2015-02-05T00:00:00"/>
+    <n v="223.5"/>
+    <s v="EN"/>
+    <n v="0"/>
+    <s v="l2"/>
+    <x v="2"/>
+  </r>
+  <r>
+    <d v="2015-02-05T00:00:00"/>
+    <n v="223.5"/>
+    <s v="EN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="2"/>
+  </r>
+  <r>
+    <d v="2015-02-05T00:00:00"/>
+    <n v="223.5"/>
+    <s v="EN"/>
+    <n v="0"/>
+    <s v="l1"/>
+    <x v="2"/>
+  </r>
+  <r>
+    <d v="2015-02-05T00:00:00"/>
+    <n v="223.5"/>
+    <s v="EN"/>
+    <n v="8"/>
+    <s v="l1"/>
+    <x v="2"/>
+  </r>
+  <r>
+    <d v="2015-02-05T00:00:00"/>
+    <n v="218.2"/>
+    <s v="SVR"/>
+    <n v="8"/>
+    <s v="l1"/>
+    <x v="2"/>
+  </r>
+  <r>
+    <d v="2015-02-06T00:00:00"/>
+    <n v="208.5"/>
+    <s v="EN"/>
+    <n v="0"/>
+    <s v="l2"/>
+    <x v="3"/>
+  </r>
+  <r>
+    <d v="2015-02-06T00:00:00"/>
+    <n v="208.5"/>
+    <s v="EN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="3"/>
+  </r>
+  <r>
+    <d v="2015-02-06T00:00:00"/>
+    <n v="208.5"/>
+    <s v="EN"/>
+    <n v="0"/>
+    <s v="l1"/>
+    <x v="3"/>
+  </r>
+  <r>
+    <d v="2015-02-06T00:00:00"/>
+    <n v="208.5"/>
+    <s v="EN"/>
+    <n v="8"/>
+    <s v="l1"/>
+    <x v="3"/>
+  </r>
+  <r>
+    <d v="2015-02-06T00:00:00"/>
+    <n v="212.2"/>
+    <s v="SVR"/>
+    <n v="8"/>
+    <s v="l1"/>
+    <x v="3"/>
+  </r>
+  <r>
+    <d v="2015-02-06T00:00:00"/>
+    <n v="239.9"/>
+    <s v="EN"/>
+    <n v="0"/>
+    <s v="l2"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <d v="2015-02-06T00:00:00"/>
+    <n v="239.9"/>
+    <s v="EN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <d v="2015-02-06T00:00:00"/>
+    <n v="229.2"/>
+    <s v="EN"/>
+    <n v="0"/>
+    <s v="l1"/>
+    <x v="5"/>
+  </r>
+  <r>
+    <d v="2015-02-06T00:00:00"/>
+    <n v="239.9"/>
+    <s v="EN"/>
+    <n v="8"/>
+    <s v="l1"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <d v="2015-02-06T00:00:00"/>
+    <n v="213.7"/>
+    <s v="SVR"/>
+    <n v="8"/>
+    <s v="l1"/>
+    <x v="3"/>
+  </r>
+  <r>
+    <d v="2015-02-07T00:00:00"/>
+    <n v="232.5"/>
+    <s v="EN"/>
+    <n v="0"/>
+    <s v="l2"/>
+    <x v="5"/>
+  </r>
+  <r>
+    <d v="2015-02-07T00:00:00"/>
+    <n v="188.4"/>
+    <s v="EN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="7"/>
+  </r>
+  <r>
+    <d v="2015-02-07T00:00:00"/>
+    <n v="232.5"/>
+    <s v="EN"/>
+    <n v="0"/>
+    <s v="l1"/>
+    <x v="5"/>
+  </r>
+  <r>
+    <d v="2015-02-07T00:00:00"/>
+    <n v="188.4"/>
+    <s v="EN"/>
+    <n v="8"/>
+    <s v="l1"/>
+    <x v="7"/>
+  </r>
+  <r>
+    <d v="2015-02-07T00:00:00"/>
+    <n v="244"/>
+    <s v="SVR"/>
+    <n v="8"/>
+    <s v="l1"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <d v="2015-02-07T00:00:00"/>
+    <n v="248.9"/>
+    <s v="NN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="6"/>
+  </r>
+  <r>
+    <d v="2015-02-08T00:00:00"/>
+    <n v="159.4"/>
+    <s v="EN"/>
+    <n v="0"/>
+    <s v="l2"/>
+    <x v="9"/>
+  </r>
+  <r>
+    <d v="2015-02-08T00:00:00"/>
+    <n v="159.4"/>
+    <s v="EN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="9"/>
+  </r>
+  <r>
+    <d v="2015-02-08T00:00:00"/>
+    <n v="159.4"/>
+    <s v="EN"/>
+    <n v="0"/>
+    <s v="l1"/>
+    <x v="9"/>
+  </r>
+  <r>
+    <d v="2015-02-08T00:00:00"/>
+    <n v="187.1"/>
+    <s v="EN"/>
+    <n v="8"/>
+    <s v="l1"/>
+    <x v="7"/>
+  </r>
+  <r>
+    <d v="2015-02-08T00:00:00"/>
+    <n v="194.6"/>
+    <s v="SVR"/>
+    <n v="8"/>
+    <s v="l1"/>
+    <x v="7"/>
+  </r>
+  <r>
+    <d v="2015-02-08T00:00:00"/>
+    <n v="176.7"/>
+    <s v="NN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="10"/>
+  </r>
+  <r>
+    <d v="2015-02-09T00:00:00"/>
+    <n v="210.6"/>
+    <s v="EN"/>
+    <n v="0"/>
+    <s v="l2"/>
+    <x v="3"/>
+  </r>
+  <r>
+    <d v="2015-02-09T00:00:00"/>
+    <n v="203.9"/>
+    <s v="EN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="12"/>
+  </r>
+  <r>
+    <d v="2015-02-09T00:00:00"/>
+    <n v="221.5"/>
+    <s v="EN"/>
+    <n v="0"/>
+    <s v="l1"/>
+    <x v="2"/>
+  </r>
+  <r>
+    <d v="2015-02-09T00:00:00"/>
+    <n v="221.5"/>
+    <s v="EN"/>
+    <n v="8"/>
+    <s v="l1"/>
+    <x v="2"/>
+  </r>
+  <r>
+    <d v="2015-02-09T00:00:00"/>
+    <n v="218.5"/>
+    <s v="SVR"/>
+    <n v="8"/>
+    <s v="l1"/>
+    <x v="2"/>
+  </r>
+  <r>
+    <d v="2015-02-09T00:00:00"/>
+    <n v="199.8"/>
+    <s v="NN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="12"/>
+  </r>
+  <r>
+    <d v="2015-02-11T00:00:00"/>
+    <n v="205.5"/>
+    <s v="EN"/>
+    <n v="0"/>
+    <s v="l2"/>
+    <x v="3"/>
+  </r>
+  <r>
+    <d v="2015-02-11T00:00:00"/>
+    <n v="222"/>
+    <s v="EN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="2"/>
+  </r>
+  <r>
+    <d v="2015-02-11T00:00:00"/>
+    <n v="203.3"/>
+    <s v="SVR"/>
+    <n v="8"/>
+    <s v="l1"/>
+    <x v="12"/>
+  </r>
+  <r>
+    <d v="2015-02-11T00:00:00"/>
+    <n v="219.4"/>
+    <s v="NN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="2"/>
   </r>
 </pivotCacheRecords>
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable1" cacheId="12" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="4" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="4" indent="0" outline="1" outlineData="1" gridDropZones="1" multipleFieldFilters="0">
-  <location ref="A3:B19" firstHeaderRow="2" firstDataRow="2" firstDataCol="1"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable1" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="4" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="4" indent="0" outline="1" outlineData="1" gridDropZones="1" multipleFieldFilters="0">
+  <location ref="A3:B20" firstHeaderRow="2" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="6">
     <pivotField numFmtId="14" showAll="0"/>
     <pivotField dataField="1" showAll="0"/>
@@ -1772,7 +2355,7 @@
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField axis="axisRow" showAll="0">
-      <items count="15">
+      <items count="16">
         <item x="13"/>
         <item x="9"/>
         <item x="1"/>
@@ -1787,6 +2370,7 @@
         <item x="4"/>
         <item x="11"/>
         <item x="8"/>
+        <item x="14"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -1794,7 +2378,7 @@
   <rowFields count="1">
     <field x="5"/>
   </rowFields>
-  <rowItems count="15">
+  <rowItems count="16">
     <i>
       <x/>
     </i>
@@ -1836,6 +2420,9 @@
     </i>
     <i>
       <x v="13"/>
+    </i>
+    <i>
+      <x v="14"/>
     </i>
     <i t="grand">
       <x/>
@@ -2889,7 +3476,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A3:W19"/>
+  <dimension ref="A3:W20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0"/>
   <cols>
     <col min="1" max="1" width="13.1640625" customWidth="1"/>
@@ -2910,7 +3497,7 @@
       </c>
       <c r="W3">
         <f>_xlfn.NORM.DIST(V3,Sheet4!$J$2,Sheet4!$J$3,FALSE)</f>
-        <v>1.3191266484266163E-3</v>
+        <v>1.1393633168699394E-3</v>
       </c>
     </row>
     <row r="4" spans="1:23">
@@ -2925,7 +3512,7 @@
       </c>
       <c r="W4">
         <f>_xlfn.NORM.DIST(V4,Sheet4!$J$2,Sheet4!$J$3,FALSE)</f>
-        <v>2.4859306893578424E-3</v>
+        <v>2.2390141961175767E-3</v>
       </c>
     </row>
     <row r="5" spans="1:23">
@@ -2940,7 +3527,7 @@
       </c>
       <c r="W5">
         <f>_xlfn.NORM.DIST(V5,Sheet4!$J$2,Sheet4!$J$3,FALSE)</f>
-        <v>4.225175141815243E-3</v>
+        <v>3.9460392509322595E-3</v>
       </c>
     </row>
     <row r="6" spans="1:23">
@@ -2948,14 +3535,14 @@
         <v>160</v>
       </c>
       <c r="B6" s="18">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="V6">
         <v>180</v>
       </c>
       <c r="W6">
         <f>_xlfn.NORM.DIST(V6,Sheet4!$J$2,Sheet4!$J$3,FALSE)</f>
-        <v>6.4766972164444301E-3</v>
+        <v>6.2370021495231475E-3</v>
       </c>
     </row>
     <row r="7" spans="1:23">
@@ -2970,7 +3557,7 @@
       </c>
       <c r="W7">
         <f>_xlfn.NORM.DIST(V7,Sheet4!$J$2,Sheet4!$J$3,FALSE)</f>
-        <v>8.9539703302276355E-3</v>
+        <v>8.8409783254578614E-3</v>
       </c>
     </row>
     <row r="8" spans="1:23">
@@ -2978,14 +3565,14 @@
         <v>180</v>
       </c>
       <c r="B8" s="18">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="V8">
         <v>200</v>
       </c>
       <c r="W8">
         <f>_xlfn.NORM.DIST(V8,Sheet4!$J$2,Sheet4!$J$3,FALSE)</f>
-        <v>1.1164284259627054E-2</v>
+        <v>1.1239181825555446E-2</v>
       </c>
     </row>
     <row r="9" spans="1:23">
@@ -2993,14 +3580,14 @@
         <v>190</v>
       </c>
       <c r="B9" s="18">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="V9">
         <v>210</v>
       </c>
       <c r="W9">
         <f>_xlfn.NORM.DIST(V9,Sheet4!$J$2,Sheet4!$J$3,FALSE)</f>
-        <v>1.2554496464711684E-2</v>
+        <v>1.2813831471045038E-2</v>
       </c>
     </row>
     <row r="10" spans="1:23">
@@ -3008,14 +3595,14 @@
         <v>200</v>
       </c>
       <c r="B10" s="18">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="V10">
         <v>220</v>
       </c>
       <c r="W10">
         <f>_xlfn.NORM.DIST(V10,Sheet4!$J$2,Sheet4!$J$3,FALSE)</f>
-        <v>1.2732711237242653E-2</v>
+        <v>1.3101869145774273E-2</v>
       </c>
     </row>
     <row r="11" spans="1:23">
@@ -3023,14 +3610,14 @@
         <v>210</v>
       </c>
       <c r="B11" s="18">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="V11">
         <v>230</v>
       </c>
       <c r="W11">
         <f>_xlfn.NORM.DIST(V11,Sheet4!$J$2,Sheet4!$J$3,FALSE)</f>
-        <v>1.1646506121258945E-2</v>
+        <v>1.2014271630391963E-2</v>
       </c>
     </row>
     <row r="12" spans="1:23">
@@ -3038,14 +3625,14 @@
         <v>220</v>
       </c>
       <c r="B12" s="18">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="V12">
         <v>240</v>
       </c>
       <c r="W12">
         <f>_xlfn.NORM.DIST(V12,Sheet4!$J$2,Sheet4!$J$3,FALSE)</f>
-        <v>9.607792319486835E-3</v>
+        <v>9.8803328398412143E-3</v>
       </c>
     </row>
     <row r="13" spans="1:23">
@@ -3053,14 +3640,14 @@
         <v>230</v>
       </c>
       <c r="B13" s="18">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="V13">
         <v>250</v>
       </c>
       <c r="W13">
         <f>_xlfn.NORM.DIST(V13,Sheet4!$J$2,Sheet4!$J$3,FALSE)</f>
-        <v>7.1483322926474855E-3</v>
+        <v>7.2871153216842394E-3</v>
       </c>
     </row>
     <row r="14" spans="1:23">
@@ -3068,14 +3655,14 @@
         <v>240</v>
       </c>
       <c r="B14" s="18">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="V14">
         <v>260</v>
       </c>
       <c r="W14">
         <f>_xlfn.NORM.DIST(V14,Sheet4!$J$2,Sheet4!$J$3,FALSE)</f>
-        <v>4.7966611154132387E-3</v>
+        <v>4.8200289779360391E-3</v>
       </c>
     </row>
     <row r="15" spans="1:23">
@@ -3083,14 +3670,14 @@
         <v>250</v>
       </c>
       <c r="B15" s="18">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="V15">
         <v>270</v>
       </c>
       <c r="W15">
         <f>_xlfn.NORM.DIST(V15,Sheet4!$J$2,Sheet4!$J$3,FALSE)</f>
-        <v>2.9028628589170603E-3</v>
+        <v>2.8592596478103334E-3</v>
       </c>
     </row>
     <row r="16" spans="1:23">
@@ -3105,18 +3692,25 @@
       </c>
       <c r="W16">
         <f>_xlfn.NORM.DIST(V16,Sheet4!$J$2,Sheet4!$J$3,FALSE)</f>
-        <v>1.5844085565882061E-3</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2">
+        <v>1.5211340235296864E-3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:23">
       <c r="A17" s="17">
         <v>270</v>
       </c>
       <c r="B17" s="18">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2">
+        <v>9</v>
+      </c>
+      <c r="V17">
+        <v>290</v>
+      </c>
+      <c r="W17">
+        <f>_xlfn.NORM.DIST(V17,Sheet4!$J$2,Sheet4!$J$3,FALSE)</f>
+        <v>7.2575711948566013E-4</v>
+      </c>
+    </row>
+    <row r="18" spans="1:23">
       <c r="A18" s="17">
         <v>280</v>
       </c>
@@ -3124,12 +3718,20 @@
         <v>2</v>
       </c>
     </row>
-    <row r="19" spans="1:2">
-      <c r="A19" s="17" t="s">
+    <row r="19" spans="1:23">
+      <c r="A19" s="17">
+        <v>290</v>
+      </c>
+      <c r="B19" s="18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:23">
+      <c r="A20" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="B19" s="18">
-        <v>100</v>
+      <c r="B20" s="18">
+        <v>147</v>
       </c>
     </row>
   </sheetData>
@@ -3200,7 +3802,7 @@
       </c>
       <c r="J2">
         <f>AVERAGE(B:B)</f>
-        <v>216.36500000000004</v>
+        <v>217.04149659863958</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="18">
@@ -3228,7 +3830,7 @@
       </c>
       <c r="J3">
         <f>_xlfn.STDEV.S(B:B)</f>
-        <v>31.119049266851356</v>
+        <v>30.304506748198964</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="18">
@@ -5647,7 +6249,9 @@
       <c r="A102" s="1">
         <v>42038</v>
       </c>
-      <c r="B102" s="19"/>
+      <c r="B102" s="19">
+        <v>272.2</v>
+      </c>
       <c r="C102" s="20" t="s">
         <v>12</v>
       </c>
@@ -5656,6 +6260,10 @@
       </c>
       <c r="E102" s="19" t="s">
         <v>13</v>
+      </c>
+      <c r="F102">
+        <f>ROUND(B102/10,0)*10</f>
+        <v>270</v>
       </c>
       <c r="G102" s="22" t="s">
         <v>39</v>
@@ -5668,7 +6276,9 @@
       <c r="A103" s="1">
         <v>42038</v>
       </c>
-      <c r="B103" s="19"/>
+      <c r="B103" s="19">
+        <v>272.2</v>
+      </c>
       <c r="C103" s="20" t="s">
         <v>12</v>
       </c>
@@ -5677,6 +6287,10 @@
       </c>
       <c r="E103" s="19" t="s">
         <v>13</v>
+      </c>
+      <c r="F103">
+        <f t="shared" ref="F103:F105" si="3">ROUND(B103/10,0)*10</f>
+        <v>270</v>
       </c>
       <c r="G103" s="22" t="s">
         <v>39</v>
@@ -5689,7 +6303,9 @@
       <c r="A104" s="1">
         <v>42038</v>
       </c>
-      <c r="B104" s="19"/>
+      <c r="B104" s="19">
+        <v>272.2</v>
+      </c>
       <c r="C104" s="20" t="s">
         <v>12</v>
       </c>
@@ -5698,6 +6314,10 @@
       </c>
       <c r="E104" s="19" t="s">
         <v>19</v>
+      </c>
+      <c r="F104">
+        <f t="shared" si="3"/>
+        <v>270</v>
       </c>
       <c r="G104" s="22" t="s">
         <v>39</v>
@@ -5710,7 +6330,9 @@
       <c r="A105" s="1">
         <v>42038</v>
       </c>
-      <c r="B105" s="19"/>
+      <c r="B105" s="19">
+        <v>272.2</v>
+      </c>
       <c r="C105" s="20" t="s">
         <v>12</v>
       </c>
@@ -5719,6 +6341,10 @@
       </c>
       <c r="E105" s="19" t="s">
         <v>19</v>
+      </c>
+      <c r="F105">
+        <f t="shared" si="3"/>
+        <v>270</v>
       </c>
       <c r="G105" s="22" t="s">
         <v>39</v>
@@ -5731,7 +6357,9 @@
       <c r="A106" s="1">
         <v>42038</v>
       </c>
-      <c r="B106" s="19"/>
+      <c r="B106" s="19">
+        <v>291.10000000000002</v>
+      </c>
       <c r="C106" s="20" t="s">
         <v>20</v>
       </c>
@@ -5741,6 +6369,10 @@
       <c r="E106" s="19" t="s">
         <v>19</v>
       </c>
+      <c r="F106">
+        <f t="shared" ref="F106:F148" si="4">ROUND(B106/10,0)*10</f>
+        <v>290</v>
+      </c>
       <c r="G106" s="22" t="s">
         <v>38</v>
       </c>
@@ -5748,272 +6380,1256 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:9">
+    <row r="107" spans="1:9" ht="25">
+      <c r="A107" s="1">
+        <v>42039</v>
+      </c>
+      <c r="B107" s="19">
+        <v>213</v>
+      </c>
+      <c r="C107" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D107" s="20">
+        <v>0</v>
+      </c>
+      <c r="E107" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F107">
+        <f t="shared" si="4"/>
+        <v>210</v>
+      </c>
+      <c r="G107" s="22" t="s">
+        <v>44</v>
+      </c>
       <c r="I107">
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="1:9">
+    <row r="108" spans="1:9" ht="25">
+      <c r="A108" s="1">
+        <v>42039</v>
+      </c>
+      <c r="B108" s="19">
+        <v>229.7</v>
+      </c>
+      <c r="C108" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D108" s="20">
+        <v>8</v>
+      </c>
+      <c r="E108" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F108">
+        <f t="shared" si="4"/>
+        <v>230</v>
+      </c>
+      <c r="G108" s="22" t="s">
+        <v>43</v>
+      </c>
       <c r="I108">
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="1:9">
+    <row r="109" spans="1:9" ht="25">
+      <c r="A109" s="1">
+        <v>42039</v>
+      </c>
+      <c r="B109" s="19">
+        <v>199.2</v>
+      </c>
+      <c r="C109" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D109" s="20">
+        <v>0</v>
+      </c>
+      <c r="E109" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F109">
+        <f t="shared" si="4"/>
+        <v>200</v>
+      </c>
+      <c r="G109" s="22" t="s">
+        <v>42</v>
+      </c>
       <c r="I109">
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:9">
+    <row r="110" spans="1:9" ht="25">
+      <c r="A110" s="1">
+        <v>42039</v>
+      </c>
+      <c r="B110" s="19">
+        <v>210.5</v>
+      </c>
+      <c r="C110" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D110" s="20">
+        <v>8</v>
+      </c>
+      <c r="E110" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F110">
+        <f t="shared" si="4"/>
+        <v>210</v>
+      </c>
+      <c r="G110" s="22" t="s">
+        <v>41</v>
+      </c>
       <c r="I110">
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="1:9">
+    <row r="111" spans="1:9" ht="25">
+      <c r="A111" s="1">
+        <v>42039</v>
+      </c>
+      <c r="B111" s="19">
+        <v>218</v>
+      </c>
+      <c r="C111" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="D111" s="20">
+        <v>8</v>
+      </c>
+      <c r="E111" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F111">
+        <f t="shared" si="4"/>
+        <v>220</v>
+      </c>
+      <c r="G111" s="22" t="s">
+        <v>40</v>
+      </c>
       <c r="I111">
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:9">
+    <row r="112" spans="1:9" ht="25">
+      <c r="A112" s="1">
+        <v>42040</v>
+      </c>
+      <c r="B112" s="19">
+        <v>223.5</v>
+      </c>
+      <c r="C112" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D112" s="20">
+        <v>0</v>
+      </c>
+      <c r="E112" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F112">
+        <f t="shared" si="4"/>
+        <v>220</v>
+      </c>
+      <c r="G112" s="22" t="s">
+        <v>46</v>
+      </c>
       <c r="I112">
         <v>0</v>
       </c>
     </row>
-    <row r="113" spans="9:9">
+    <row r="113" spans="1:9" ht="25">
+      <c r="A113" s="1">
+        <v>42040</v>
+      </c>
+      <c r="B113" s="19">
+        <v>223.5</v>
+      </c>
+      <c r="C113" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D113" s="20">
+        <v>8</v>
+      </c>
+      <c r="E113" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F113">
+        <f t="shared" si="4"/>
+        <v>220</v>
+      </c>
+      <c r="G113" s="22" t="s">
+        <v>46</v>
+      </c>
       <c r="I113">
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="9:9">
+    <row r="114" spans="1:9" ht="25">
+      <c r="A114" s="1">
+        <v>42040</v>
+      </c>
+      <c r="B114" s="19">
+        <v>223.5</v>
+      </c>
+      <c r="C114" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D114" s="20">
+        <v>0</v>
+      </c>
+      <c r="E114" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F114">
+        <f t="shared" si="4"/>
+        <v>220</v>
+      </c>
+      <c r="G114" s="22" t="s">
+        <v>46</v>
+      </c>
       <c r="I114">
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="9:9">
+    <row r="115" spans="1:9" ht="25">
+      <c r="A115" s="1">
+        <v>42040</v>
+      </c>
+      <c r="B115" s="19">
+        <v>223.5</v>
+      </c>
+      <c r="C115" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D115" s="20">
+        <v>8</v>
+      </c>
+      <c r="E115" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F115">
+        <f t="shared" si="4"/>
+        <v>220</v>
+      </c>
+      <c r="G115" s="22" t="s">
+        <v>46</v>
+      </c>
       <c r="I115">
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="9:9">
+    <row r="116" spans="1:9" ht="25">
+      <c r="A116" s="1">
+        <v>42040</v>
+      </c>
+      <c r="B116" s="19">
+        <v>218.2</v>
+      </c>
+      <c r="C116" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="D116" s="20">
+        <v>8</v>
+      </c>
+      <c r="E116" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F116">
+        <f t="shared" si="4"/>
+        <v>220</v>
+      </c>
+      <c r="G116" s="22" t="s">
+        <v>45</v>
+      </c>
       <c r="I116">
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="9:9">
+    <row r="117" spans="1:9" ht="25">
+      <c r="A117" s="1">
+        <v>42041</v>
+      </c>
+      <c r="B117">
+        <v>208.5</v>
+      </c>
+      <c r="C117" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D117" s="20">
+        <v>0</v>
+      </c>
+      <c r="E117" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F117">
+        <f t="shared" si="4"/>
+        <v>210</v>
+      </c>
+      <c r="G117" s="22" t="s">
+        <v>48</v>
+      </c>
       <c r="I117">
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="9:9">
+    <row r="118" spans="1:9" ht="25">
+      <c r="A118" s="1">
+        <v>42041</v>
+      </c>
+      <c r="B118">
+        <v>208.5</v>
+      </c>
+      <c r="C118" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D118" s="20">
+        <v>8</v>
+      </c>
+      <c r="E118" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F118">
+        <f t="shared" si="4"/>
+        <v>210</v>
+      </c>
+      <c r="G118" s="22" t="s">
+        <v>48</v>
+      </c>
       <c r="I118">
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="9:9">
+    <row r="119" spans="1:9" ht="25">
+      <c r="A119" s="1">
+        <v>42041</v>
+      </c>
+      <c r="B119">
+        <v>208.5</v>
+      </c>
+      <c r="C119" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D119" s="20">
+        <v>0</v>
+      </c>
+      <c r="E119" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F119">
+        <f t="shared" si="4"/>
+        <v>210</v>
+      </c>
+      <c r="G119" s="22" t="s">
+        <v>48</v>
+      </c>
       <c r="I119">
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="9:9">
+    <row r="120" spans="1:9" ht="25">
+      <c r="A120" s="1">
+        <v>42041</v>
+      </c>
+      <c r="B120">
+        <v>208.5</v>
+      </c>
+      <c r="C120" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D120" s="20">
+        <v>8</v>
+      </c>
+      <c r="E120" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F120">
+        <f t="shared" si="4"/>
+        <v>210</v>
+      </c>
+      <c r="G120" s="22" t="s">
+        <v>48</v>
+      </c>
       <c r="I120">
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="9:9">
+    <row r="121" spans="1:9" ht="25">
+      <c r="A121" s="1">
+        <v>42041</v>
+      </c>
+      <c r="B121">
+        <v>212.2</v>
+      </c>
+      <c r="C121" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="D121" s="20">
+        <v>8</v>
+      </c>
+      <c r="E121" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F121">
+        <f t="shared" si="4"/>
+        <v>210</v>
+      </c>
+      <c r="G121" s="22" t="s">
+        <v>47</v>
+      </c>
       <c r="I121">
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="9:9">
+    <row r="122" spans="1:9" ht="25">
+      <c r="A122" s="1">
+        <v>42041</v>
+      </c>
+      <c r="B122">
+        <v>239.9</v>
+      </c>
+      <c r="C122" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D122" s="20">
+        <v>0</v>
+      </c>
+      <c r="E122" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F122">
+        <f t="shared" si="4"/>
+        <v>240</v>
+      </c>
+      <c r="G122" s="22" t="s">
+        <v>50</v>
+      </c>
       <c r="I122">
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="9:9">
+    <row r="123" spans="1:9" ht="25">
+      <c r="A123" s="1">
+        <v>42041</v>
+      </c>
+      <c r="B123">
+        <v>239.9</v>
+      </c>
+      <c r="C123" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D123" s="20">
+        <v>8</v>
+      </c>
+      <c r="E123" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F123">
+        <f t="shared" si="4"/>
+        <v>240</v>
+      </c>
+      <c r="G123" s="22" t="s">
+        <v>50</v>
+      </c>
       <c r="I123">
         <v>0</v>
       </c>
     </row>
-    <row r="124" spans="9:9">
+    <row r="124" spans="1:9" ht="25">
+      <c r="A124" s="1">
+        <v>42041</v>
+      </c>
+      <c r="B124">
+        <v>229.2</v>
+      </c>
+      <c r="C124" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D124" s="20">
+        <v>0</v>
+      </c>
+      <c r="E124" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F124">
+        <f t="shared" si="4"/>
+        <v>230</v>
+      </c>
+      <c r="G124" s="22" t="s">
+        <v>51</v>
+      </c>
       <c r="I124">
         <v>0</v>
       </c>
     </row>
-    <row r="125" spans="9:9">
+    <row r="125" spans="1:9" ht="25">
+      <c r="A125" s="1">
+        <v>42041</v>
+      </c>
+      <c r="B125">
+        <v>239.9</v>
+      </c>
+      <c r="C125" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D125" s="20">
+        <v>8</v>
+      </c>
+      <c r="E125" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F125">
+        <f t="shared" si="4"/>
+        <v>240</v>
+      </c>
+      <c r="G125" s="22" t="s">
+        <v>50</v>
+      </c>
       <c r="I125">
         <v>0</v>
       </c>
     </row>
-    <row r="126" spans="9:9">
+    <row r="126" spans="1:9" ht="25">
+      <c r="A126" s="1">
+        <v>42041</v>
+      </c>
+      <c r="B126">
+        <v>213.7</v>
+      </c>
+      <c r="C126" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="D126" s="20">
+        <v>8</v>
+      </c>
+      <c r="E126" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F126">
+        <f t="shared" si="4"/>
+        <v>210</v>
+      </c>
+      <c r="G126" s="22" t="s">
+        <v>49</v>
+      </c>
       <c r="I126">
         <v>0</v>
       </c>
     </row>
-    <row r="127" spans="9:9">
+    <row r="127" spans="1:9" ht="25">
+      <c r="A127" s="1">
+        <v>42042</v>
+      </c>
+      <c r="B127">
+        <v>232.5</v>
+      </c>
+      <c r="C127" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D127" s="20">
+        <v>0</v>
+      </c>
+      <c r="E127" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F127">
+        <f t="shared" si="4"/>
+        <v>230</v>
+      </c>
+      <c r="G127" s="22" t="s">
+        <v>52</v>
+      </c>
       <c r="I127">
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="9:9">
+    <row r="128" spans="1:9" ht="25">
+      <c r="A128" s="1">
+        <v>42042</v>
+      </c>
+      <c r="B128">
+        <v>188.4</v>
+      </c>
+      <c r="C128" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D128" s="20">
+        <v>8</v>
+      </c>
+      <c r="E128" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F128">
+        <f t="shared" si="4"/>
+        <v>190</v>
+      </c>
+      <c r="G128" s="22" t="s">
+        <v>53</v>
+      </c>
       <c r="I128">
         <v>0</v>
       </c>
     </row>
-    <row r="129" spans="9:9">
+    <row r="129" spans="1:9" ht="25">
+      <c r="A129" s="1">
+        <v>42042</v>
+      </c>
+      <c r="B129">
+        <v>232.5</v>
+      </c>
+      <c r="C129" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D129" s="20">
+        <v>0</v>
+      </c>
+      <c r="E129" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F129">
+        <f t="shared" si="4"/>
+        <v>230</v>
+      </c>
+      <c r="G129" s="22" t="s">
+        <v>52</v>
+      </c>
       <c r="I129">
         <v>0</v>
       </c>
     </row>
-    <row r="130" spans="9:9">
+    <row r="130" spans="1:9" ht="25">
+      <c r="A130" s="1">
+        <v>42042</v>
+      </c>
+      <c r="B130">
+        <v>188.4</v>
+      </c>
+      <c r="C130" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D130" s="20">
+        <v>8</v>
+      </c>
+      <c r="E130" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F130">
+        <f t="shared" si="4"/>
+        <v>190</v>
+      </c>
+      <c r="G130" s="22" t="s">
+        <v>53</v>
+      </c>
       <c r="I130">
         <v>0</v>
       </c>
     </row>
-    <row r="131" spans="9:9">
+    <row r="131" spans="1:9" ht="25">
+      <c r="A131" s="1">
+        <v>42042</v>
+      </c>
+      <c r="B131">
+        <v>244</v>
+      </c>
+      <c r="C131" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="D131" s="20">
+        <v>8</v>
+      </c>
+      <c r="E131" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F131">
+        <f t="shared" si="4"/>
+        <v>240</v>
+      </c>
+      <c r="G131" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="I131">
         <v>0</v>
       </c>
     </row>
-    <row r="132" spans="9:9">
+    <row r="132" spans="1:9" ht="25">
+      <c r="A132" s="1">
+        <v>42042</v>
+      </c>
+      <c r="B132">
+        <v>248.9</v>
+      </c>
+      <c r="C132" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="D132" s="20">
+        <v>8</v>
+      </c>
+      <c r="E132" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F132">
+        <f t="shared" si="4"/>
+        <v>250</v>
+      </c>
+      <c r="G132" s="22" t="s">
+        <v>55</v>
+      </c>
       <c r="I132">
         <v>0</v>
       </c>
     </row>
-    <row r="133" spans="9:9">
+    <row r="133" spans="1:9" ht="25">
+      <c r="A133" s="1">
+        <v>42043</v>
+      </c>
+      <c r="B133">
+        <v>159.4</v>
+      </c>
+      <c r="C133" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D133" s="20">
+        <v>0</v>
+      </c>
+      <c r="E133" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F133">
+        <f t="shared" si="4"/>
+        <v>160</v>
+      </c>
+      <c r="G133" s="22" t="s">
+        <v>60</v>
+      </c>
       <c r="I133">
         <v>0</v>
       </c>
     </row>
-    <row r="134" spans="9:9">
+    <row r="134" spans="1:9" ht="25">
+      <c r="A134" s="1">
+        <v>42043</v>
+      </c>
+      <c r="B134">
+        <v>159.4</v>
+      </c>
+      <c r="C134" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D134" s="20">
+        <v>8</v>
+      </c>
+      <c r="E134" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F134">
+        <f t="shared" si="4"/>
+        <v>160</v>
+      </c>
+      <c r="G134" s="22" t="s">
+        <v>60</v>
+      </c>
       <c r="I134">
         <v>0</v>
       </c>
     </row>
-    <row r="135" spans="9:9">
+    <row r="135" spans="1:9" ht="25">
+      <c r="A135" s="1">
+        <v>42043</v>
+      </c>
+      <c r="B135">
+        <v>159.4</v>
+      </c>
+      <c r="C135" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D135" s="20">
+        <v>0</v>
+      </c>
+      <c r="E135" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F135">
+        <f t="shared" si="4"/>
+        <v>160</v>
+      </c>
+      <c r="G135" s="22" t="s">
+        <v>60</v>
+      </c>
       <c r="I135">
         <v>0</v>
       </c>
     </row>
-    <row r="136" spans="9:9">
+    <row r="136" spans="1:9" ht="25">
+      <c r="A136" s="1">
+        <v>42043</v>
+      </c>
+      <c r="B136">
+        <v>187.1</v>
+      </c>
+      <c r="C136" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D136" s="20">
+        <v>8</v>
+      </c>
+      <c r="E136" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F136">
+        <f t="shared" si="4"/>
+        <v>190</v>
+      </c>
+      <c r="G136" s="22" t="s">
+        <v>59</v>
+      </c>
       <c r="I136">
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="9:9">
+    <row r="137" spans="1:9" ht="25">
+      <c r="A137" s="1">
+        <v>42043</v>
+      </c>
+      <c r="B137">
+        <v>194.6</v>
+      </c>
+      <c r="C137" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="D137" s="20">
+        <v>8</v>
+      </c>
+      <c r="E137" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F137">
+        <f t="shared" si="4"/>
+        <v>190</v>
+      </c>
+      <c r="G137" s="22" t="s">
+        <v>58</v>
+      </c>
       <c r="I137">
         <v>0</v>
       </c>
     </row>
-    <row r="138" spans="9:9">
+    <row r="138" spans="1:9" ht="25">
+      <c r="A138" s="1">
+        <v>42043</v>
+      </c>
+      <c r="B138">
+        <v>176.7</v>
+      </c>
+      <c r="C138" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="D138" s="20">
+        <v>8</v>
+      </c>
+      <c r="E138" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F138">
+        <f t="shared" si="4"/>
+        <v>180</v>
+      </c>
+      <c r="G138" s="22" t="s">
+        <v>57</v>
+      </c>
       <c r="I138">
         <v>0</v>
       </c>
     </row>
-    <row r="139" spans="9:9">
+    <row r="139" spans="1:9" ht="25">
+      <c r="A139" s="1">
+        <v>42044</v>
+      </c>
+      <c r="B139">
+        <v>210.6</v>
+      </c>
+      <c r="C139" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D139" s="20">
+        <v>0</v>
+      </c>
+      <c r="E139" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F139">
+        <f t="shared" si="4"/>
+        <v>210</v>
+      </c>
+      <c r="G139" s="22" t="s">
+        <v>62</v>
+      </c>
       <c r="I139">
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="9:9">
+    <row r="140" spans="1:9" ht="25">
+      <c r="A140" s="1">
+        <v>42044</v>
+      </c>
+      <c r="B140">
+        <v>203.9</v>
+      </c>
+      <c r="C140" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D140" s="20">
+        <v>8</v>
+      </c>
+      <c r="E140" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F140">
+        <f t="shared" si="4"/>
+        <v>200</v>
+      </c>
+      <c r="G140" s="22" t="s">
+        <v>63</v>
+      </c>
       <c r="I140">
         <v>0</v>
       </c>
     </row>
-    <row r="141" spans="9:9">
+    <row r="141" spans="1:9" ht="25">
+      <c r="A141" s="1">
+        <v>42044</v>
+      </c>
+      <c r="B141">
+        <v>221.5</v>
+      </c>
+      <c r="C141" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D141" s="20">
+        <v>0</v>
+      </c>
+      <c r="E141" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F141">
+        <f t="shared" si="4"/>
+        <v>220</v>
+      </c>
+      <c r="G141" s="22" t="s">
+        <v>61</v>
+      </c>
       <c r="I141">
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="9:9">
+    <row r="142" spans="1:9" ht="25">
+      <c r="A142" s="1">
+        <v>42044</v>
+      </c>
+      <c r="B142">
+        <v>221.5</v>
+      </c>
+      <c r="C142" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D142" s="20">
+        <v>8</v>
+      </c>
+      <c r="E142" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F142">
+        <f t="shared" si="4"/>
+        <v>220</v>
+      </c>
+      <c r="G142" s="22" t="s">
+        <v>61</v>
+      </c>
       <c r="I142">
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="9:9">
+    <row r="143" spans="1:9" ht="25">
+      <c r="A143" s="1">
+        <v>42044</v>
+      </c>
+      <c r="B143">
+        <v>218.5</v>
+      </c>
+      <c r="C143" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="D143" s="20">
+        <v>8</v>
+      </c>
+      <c r="E143" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F143">
+        <f t="shared" si="4"/>
+        <v>220</v>
+      </c>
+      <c r="G143" s="22" t="s">
+        <v>64</v>
+      </c>
       <c r="I143">
         <v>0</v>
       </c>
     </row>
-    <row r="144" spans="9:9">
+    <row r="144" spans="1:9" ht="25">
+      <c r="A144" s="1">
+        <v>42044</v>
+      </c>
+      <c r="B144">
+        <v>199.8</v>
+      </c>
+      <c r="C144" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="D144" s="20">
+        <v>8</v>
+      </c>
+      <c r="E144" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F144">
+        <f t="shared" si="4"/>
+        <v>200</v>
+      </c>
+      <c r="G144" s="22" t="s">
+        <v>65</v>
+      </c>
       <c r="I144">
         <v>0</v>
       </c>
     </row>
-    <row r="145" spans="9:9">
+    <row r="145" spans="1:9" ht="25">
+      <c r="A145" s="1">
+        <v>42046</v>
+      </c>
+      <c r="B145">
+        <v>205.5</v>
+      </c>
+      <c r="C145" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D145" s="20">
+        <v>0</v>
+      </c>
+      <c r="E145" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F145">
+        <f t="shared" si="4"/>
+        <v>210</v>
+      </c>
+      <c r="G145" s="22" t="s">
+        <v>69</v>
+      </c>
       <c r="I145">
         <v>0</v>
       </c>
     </row>
-    <row r="146" spans="9:9">
+    <row r="146" spans="1:9" ht="25">
+      <c r="A146" s="1">
+        <v>42046</v>
+      </c>
+      <c r="B146">
+        <v>222</v>
+      </c>
+      <c r="C146" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D146" s="20">
+        <v>8</v>
+      </c>
+      <c r="E146" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F146">
+        <f t="shared" si="4"/>
+        <v>220</v>
+      </c>
+      <c r="G146" s="22" t="s">
+        <v>68</v>
+      </c>
       <c r="I146">
         <v>0</v>
       </c>
     </row>
-    <row r="147" spans="9:9">
+    <row r="147" spans="1:9" ht="25">
+      <c r="A147" s="1">
+        <v>42046</v>
+      </c>
+      <c r="B147">
+        <v>203.3</v>
+      </c>
+      <c r="C147" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="D147" s="20">
+        <v>8</v>
+      </c>
+      <c r="E147" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F147">
+        <f t="shared" si="4"/>
+        <v>200</v>
+      </c>
+      <c r="G147" s="22" t="s">
+        <v>67</v>
+      </c>
       <c r="I147">
         <v>0</v>
       </c>
     </row>
-    <row r="148" spans="9:9">
+    <row r="148" spans="1:9" ht="25">
+      <c r="A148" s="1">
+        <v>42046</v>
+      </c>
+      <c r="B148">
+        <v>219.4</v>
+      </c>
+      <c r="C148" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="D148" s="20">
+        <v>8</v>
+      </c>
+      <c r="E148" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F148">
+        <f t="shared" si="4"/>
+        <v>220</v>
+      </c>
+      <c r="G148" s="22" t="s">
+        <v>66</v>
+      </c>
       <c r="I148">
         <v>0</v>
       </c>
     </row>
-    <row r="149" spans="9:9">
+    <row r="149" spans="1:9" ht="25">
+      <c r="A149" s="1">
+        <v>42047</v>
+      </c>
+      <c r="C149" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D149" s="20">
+        <v>0</v>
+      </c>
+      <c r="E149" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="G149" s="22" t="s">
+        <v>72</v>
+      </c>
       <c r="I149">
         <v>0</v>
       </c>
     </row>
-    <row r="150" spans="9:9">
+    <row r="150" spans="1:9" ht="25">
+      <c r="A150" s="1">
+        <v>42047</v>
+      </c>
+      <c r="C150" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D150" s="20">
+        <v>8</v>
+      </c>
+      <c r="E150" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="G150" s="22" t="s">
+        <v>72</v>
+      </c>
       <c r="I150">
         <v>0</v>
       </c>
     </row>
-    <row r="151" spans="9:9">
+    <row r="151" spans="1:9" ht="25">
+      <c r="A151" s="1">
+        <v>42047</v>
+      </c>
+      <c r="C151" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="D151" s="20">
+        <v>8</v>
+      </c>
+      <c r="E151" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="G151" s="22" t="s">
+        <v>71</v>
+      </c>
       <c r="I151">
         <v>0</v>
       </c>
     </row>
-    <row r="152" spans="9:9">
+    <row r="152" spans="1:9" ht="25">
+      <c r="A152" s="1">
+        <v>42047</v>
+      </c>
+      <c r="C152" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="D152" s="20">
+        <v>8</v>
+      </c>
+      <c r="E152" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="G152" s="22" t="s">
+        <v>70</v>
+      </c>
       <c r="I152">
         <v>0</v>
       </c>
     </row>
-    <row r="153" spans="9:9">
+    <row r="153" spans="1:9">
       <c r="I153">
         <v>0</v>
       </c>
     </row>
-    <row r="154" spans="9:9">
+    <row r="154" spans="1:9">
       <c r="I154">
         <v>0</v>
       </c>
     </row>
-    <row r="155" spans="9:9">
+    <row r="155" spans="1:9">
       <c r="I155">
         <v>0</v>
       </c>
     </row>
-    <row r="156" spans="9:9">
+    <row r="156" spans="1:9">
       <c r="I156">
         <v>0</v>
       </c>
     </row>
-    <row r="157" spans="9:9">
+    <row r="157" spans="1:9">
       <c r="I157">
         <v>0</v>
       </c>
     </row>
-    <row r="158" spans="9:9">
+    <row r="158" spans="1:9">
       <c r="I158">
         <v>0</v>
       </c>
     </row>
-    <row r="159" spans="9:9">
+    <row r="159" spans="1:9">
       <c r="I159">
         <v>0</v>
       </c>
     </row>
-    <row r="160" spans="9:9">
+    <row r="160" spans="1:9">
       <c r="I160">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
add opponent defense against position
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="24030"/>
   <workbookPr showInkAnnotation="0" hidePivotFieldList="1" autoCompressPictures="0"/>
   <bookViews>
-    <workbookView xWindow="1120" yWindow="1120" windowWidth="24480" windowHeight="14420" tabRatio="500" activeTab="2"/>
+    <workbookView xWindow="460" yWindow="0" windowWidth="23920" windowHeight="13860" tabRatio="500" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -13,7 +13,7 @@
   </sheets>
   <calcPr calcId="140000" concurrentCalc="0"/>
   <pivotCaches>
-    <pivotCache cacheId="3" r:id="rId4"/>
+    <pivotCache cacheId="61" r:id="rId4"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{7523E5D3-25F3-A5E0-1632-64F254C22452}">
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="676" uniqueCount="148">
   <si>
     <t>Date</t>
   </si>
@@ -243,6 +243,231 @@
   </si>
   <si>
     <t>S135327370</t>
+  </si>
+  <si>
+    <t>S135633033</t>
+  </si>
+  <si>
+    <t>S135633222</t>
+  </si>
+  <si>
+    <t>S135633562</t>
+  </si>
+  <si>
+    <t>S135642884</t>
+  </si>
+  <si>
+    <t>S135643140</t>
+  </si>
+  <si>
+    <t>S135643352</t>
+  </si>
+  <si>
+    <t>S135643523</t>
+  </si>
+  <si>
+    <t>S135786416</t>
+  </si>
+  <si>
+    <t>S135789672</t>
+  </si>
+  <si>
+    <t>S135789902</t>
+  </si>
+  <si>
+    <t>S135790226</t>
+  </si>
+  <si>
+    <t>S135945102</t>
+  </si>
+  <si>
+    <t>S135945252</t>
+  </si>
+  <si>
+    <t>S135945398</t>
+  </si>
+  <si>
+    <t>S135945603</t>
+  </si>
+  <si>
+    <t>S136132688</t>
+  </si>
+  <si>
+    <t>S136132888</t>
+  </si>
+  <si>
+    <t>S136133205</t>
+  </si>
+  <si>
+    <t>S136133382</t>
+  </si>
+  <si>
+    <t>S136335267</t>
+  </si>
+  <si>
+    <t>S136335373</t>
+  </si>
+  <si>
+    <t>S136555674</t>
+  </si>
+  <si>
+    <t>S136556105</t>
+  </si>
+  <si>
+    <t>S136556625</t>
+  </si>
+  <si>
+    <t>S136557018</t>
+  </si>
+  <si>
+    <t>S137216050</t>
+  </si>
+  <si>
+    <t>S137217925</t>
+  </si>
+  <si>
+    <t>S137219413</t>
+  </si>
+  <si>
+    <t>S137220812</t>
+  </si>
+  <si>
+    <t>S137813258</t>
+  </si>
+  <si>
+    <t>S137815124</t>
+  </si>
+  <si>
+    <t>S137816030</t>
+  </si>
+  <si>
+    <t>S137816721</t>
+  </si>
+  <si>
+    <t>S138054611</t>
+  </si>
+  <si>
+    <t>S138055001</t>
+  </si>
+  <si>
+    <t>S138055299</t>
+  </si>
+  <si>
+    <t>S138058281</t>
+  </si>
+  <si>
+    <t>S138058773</t>
+  </si>
+  <si>
+    <t>S138661867</t>
+  </si>
+  <si>
+    <t>S138662412</t>
+  </si>
+  <si>
+    <t>S138662833</t>
+  </si>
+  <si>
+    <t>S138663125</t>
+  </si>
+  <si>
+    <t>S139226573</t>
+  </si>
+  <si>
+    <t>S139227064</t>
+  </si>
+  <si>
+    <t>S139227520</t>
+  </si>
+  <si>
+    <t>S139786602</t>
+  </si>
+  <si>
+    <t>S139787499</t>
+  </si>
+  <si>
+    <t>S139787999</t>
+  </si>
+  <si>
+    <t>S139789020</t>
+  </si>
+  <si>
+    <t>S140434070</t>
+  </si>
+  <si>
+    <t>S140435728</t>
+  </si>
+  <si>
+    <t>S140436227</t>
+  </si>
+  <si>
+    <t>S140436647</t>
+  </si>
+  <si>
+    <t>S141472840</t>
+  </si>
+  <si>
+    <t>S141473050</t>
+  </si>
+  <si>
+    <t>S141473151</t>
+  </si>
+  <si>
+    <t>S141666776</t>
+  </si>
+  <si>
+    <t>S141669238</t>
+  </si>
+  <si>
+    <t>S141671781</t>
+  </si>
+  <si>
+    <t>S142232876</t>
+  </si>
+  <si>
+    <t>S142234181</t>
+  </si>
+  <si>
+    <t>S142235128</t>
+  </si>
+  <si>
+    <t>S142235844</t>
+  </si>
+  <si>
+    <t>S142506186</t>
+  </si>
+  <si>
+    <t>S142508476</t>
+  </si>
+  <si>
+    <t>S142738865</t>
+  </si>
+  <si>
+    <t>S142739177</t>
+  </si>
+  <si>
+    <t>S143277009</t>
+  </si>
+  <si>
+    <t>S143277516</t>
+  </si>
+  <si>
+    <t>S143278956</t>
+  </si>
+  <si>
+    <t>S143279379</t>
+  </si>
+  <si>
+    <t>S143907915</t>
+  </si>
+  <si>
+    <t>S143908791</t>
+  </si>
+  <si>
+    <t>S143909226</t>
+  </si>
+  <si>
+    <t>S143909636</t>
   </si>
 </sst>
 </file>
@@ -286,7 +511,7 @@
       <name val="Helvetica"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -329,6 +554,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -354,7 +585,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="162">
+  <cellStyleXfs count="249">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
@@ -517,8 +748,95 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
@@ -544,11 +862,12 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="162">
+  <cellStyles count="249">
     <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="4" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="6" builtinId="9" hidden="1"/>
@@ -630,6 +949,60 @@
     <cellStyle name="Followed Hyperlink" xfId="157" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="159" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="161" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="163" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="165" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="167" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="169" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="171" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="173" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="175" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="177" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="179" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="181" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="183" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="185" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="187" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="189" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="191" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="193" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="195" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="197" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="199" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="201" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="203" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="205" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="207" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="209" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="211" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="213" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="215" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="217" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="219" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="221" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="223" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="225" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="227" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="228" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="229" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="230" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="231" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="232" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="233" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="234" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="235" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="236" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="237" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="238" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="239" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="240" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="241" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="242" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="243" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="244" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="245" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="246" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="247" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="248" builtinId="9" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="3" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="5" builtinId="8" hidden="1"/>
@@ -710,6 +1083,39 @@
     <cellStyle name="Hyperlink" xfId="156" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="158" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="160" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="162" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="164" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="166" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="168" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="170" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="172" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="174" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="176" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="178" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="180" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="182" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="184" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="186" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="188" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="190" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="192" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="194" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="196" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="198" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="200" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="202" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="204" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="206" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="208" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="210" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="212" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="214" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="216" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="218" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="220" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="222" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="224" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="226" builtinId="8" hidden="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -803,43 +1209,43 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="15"/>
                 <c:pt idx="0">
-                  <c:v>1.0</c:v>
+                  <c:v>4.0</c:v>
                 </c:pt>
                 <c:pt idx="1">
+                  <c:v>7.0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>15.0</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>12.0</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>26.0</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>18.0</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>41.0</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>36.0</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>23.0</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>18.0</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>17.0</c:v>
+                </c:pt>
+                <c:pt idx="11">
                   <c:v>5.0</c:v>
                 </c:pt>
-                <c:pt idx="2">
-                  <c:v>9.0</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>6.0</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>19.0</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>6.0</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>28.0</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>20.0</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>13.0</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>11.0</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>14.0</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>3.0</c:v>
-                </c:pt>
                 <c:pt idx="12">
-                  <c:v>9.0</c:v>
+                  <c:v>10.0</c:v>
                 </c:pt>
                 <c:pt idx="13">
                   <c:v>2.0</c:v>
@@ -860,8 +1266,8 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="150"/>
-        <c:axId val="-2125646632"/>
-        <c:axId val="-2125738872"/>
+        <c:axId val="-2112807896"/>
+        <c:axId val="-2112811192"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -933,49 +1339,49 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="15"/>
                 <c:pt idx="0">
-                  <c:v>0.00113936331686994</c:v>
+                  <c:v>0.001232257656464</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.00223901419611758</c:v>
+                  <c:v>0.00247717835128003</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.00394603925093226</c:v>
+                  <c:v>0.00442119653601064</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.00623700214952315</c:v>
+                  <c:v>0.00700566168510025</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.00884097832545786</c:v>
+                  <c:v>0.00985565051328814</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.0112391818255554</c:v>
+                  <c:v>0.0123097213847046</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.012813831471045</c:v>
+                  <c:v>0.0136501664233175</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.0131018691457743</c:v>
+                  <c:v>0.0134386135061302</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.012014271630392</c:v>
+                  <c:v>0.0117462104015132</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.00988033283984121</c:v>
+                  <c:v>0.00911523526280455</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.00728711532168424</c:v>
+                  <c:v>0.00628007431684782</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.00482002897793604</c:v>
+                  <c:v>0.00384139068094988</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.00285925964781033</c:v>
+                  <c:v>0.00208611847027228</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>0.00152113402352969</c:v>
+                  <c:v>0.00100581070272385</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0.00072575711948566</c:v>
+                  <c:v>0.000430546765929341</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -992,11 +1398,11 @@
         </c:dLbls>
         <c:marker val="1"/>
         <c:smooth val="0"/>
-        <c:axId val="-2125732408"/>
-        <c:axId val="-2125741912"/>
+        <c:axId val="-2112817640"/>
+        <c:axId val="-2112814232"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="-2125732408"/>
+        <c:axId val="-2112817640"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1006,7 +1412,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="-2125741912"/>
+        <c:crossAx val="-2112814232"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1014,9 +1420,10 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="-2125741912"/>
+        <c:axId val="-2112814232"/>
         <c:scaling>
           <c:orientation val="minMax"/>
+          <c:max val="0.015"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
@@ -1025,14 +1432,15 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="-2125732408"/>
+        <c:crossAx val="-2112817640"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="-2125738872"/>
+        <c:axId val="-2112811192"/>
         <c:scaling>
           <c:orientation val="minMax"/>
+          <c:max val="45.0"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="r"/>
@@ -1040,12 +1448,12 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="-2125646632"/>
+        <c:crossAx val="-2112807896"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:catAx>
-        <c:axId val="-2125646632"/>
+        <c:axId val="-2112807896"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1055,7 +1463,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="-2125738872"/>
+        <c:crossAx val="-2112811192"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1065,7 +1473,6 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="r"/>
-      <c:layout/>
       <c:overlay val="0"/>
     </c:legend>
     <c:plotVisOnly val="1"/>
@@ -1116,16 +1523,16 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1" refreshedBy="Jesse Green" refreshedDate="42047.398584490744" createdVersion="4" refreshedVersion="4" minRefreshableVersion="3" recordCount="147">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1" refreshedBy="Jesse Green" refreshedDate="42066.385978819446" createdVersion="4" refreshedVersion="4" minRefreshableVersion="3" recordCount="235">
   <cacheSource type="worksheet">
-    <worksheetSource ref="A1:F148" sheet="Sheet4"/>
+    <worksheetSource ref="A1:F236" sheet="Sheet4"/>
   </cacheSource>
   <cacheFields count="6">
     <cacheField name="date" numFmtId="14">
-      <sharedItems containsSemiMixedTypes="0" containsNonDate="0" containsDate="1" containsString="0" minDate="2014-01-25T00:00:00" maxDate="2015-02-12T00:00:00"/>
+      <sharedItems containsSemiMixedTypes="0" containsNonDate="0" containsDate="1" containsString="0" minDate="2014-01-25T00:00:00" maxDate="2015-03-03T00:00:00"/>
     </cacheField>
     <cacheField name="score" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="152.30000000000001" maxValue="291.10000000000002"/>
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="150.5" maxValue="291.10000000000002"/>
     </cacheField>
     <cacheField name="model" numFmtId="0">
       <sharedItems/>
@@ -1165,7 +1572,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" count="147">
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" count="235">
   <r>
     <d v="2015-01-15T00:00:00"/>
     <n v="235.4"/>
@@ -2341,12 +2748,716 @@
     <n v="8"/>
     <s v="l2"/>
     <x v="2"/>
+  </r>
+  <r>
+    <d v="2015-02-12T00:00:00"/>
+    <n v="216.5"/>
+    <s v="EN"/>
+    <n v="0"/>
+    <s v="l2"/>
+    <x v="2"/>
+  </r>
+  <r>
+    <d v="2015-02-12T00:00:00"/>
+    <n v="216.5"/>
+    <s v="EN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="2"/>
+  </r>
+  <r>
+    <d v="2015-02-12T00:00:00"/>
+    <n v="166.3"/>
+    <s v="SVR"/>
+    <n v="8"/>
+    <s v="l1"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <d v="2015-02-12T00:00:00"/>
+    <n v="168"/>
+    <s v="NN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <d v="2015-02-14T00:00:00"/>
+    <n v="195.1"/>
+    <s v="EN"/>
+    <n v="0"/>
+    <s v="l2"/>
+    <x v="12"/>
+  </r>
+  <r>
+    <d v="2015-02-14T00:00:00"/>
+    <n v="222.4"/>
+    <s v="EN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="2"/>
+  </r>
+  <r>
+    <d v="2015-02-14T00:00:00"/>
+    <n v="205"/>
+    <s v="SVR"/>
+    <n v="8"/>
+    <s v="l1"/>
+    <x v="3"/>
+  </r>
+  <r>
+    <d v="2015-02-14T00:00:00"/>
+    <n v="222.4"/>
+    <s v="NN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="2"/>
+  </r>
+  <r>
+    <d v="2015-02-14T00:00:00"/>
+    <n v="200"/>
+    <s v="EN"/>
+    <n v="0"/>
+    <s v="l2"/>
+    <x v="12"/>
+  </r>
+  <r>
+    <d v="2015-02-14T00:00:00"/>
+    <n v="234.8"/>
+    <s v="EN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="5"/>
+  </r>
+  <r>
+    <d v="2015-02-14T00:00:00"/>
+    <n v="222.3"/>
+    <s v="SVR"/>
+    <n v="8"/>
+    <s v="l1"/>
+    <x v="2"/>
+  </r>
+  <r>
+    <d v="2015-02-14T00:00:00"/>
+    <n v="220.9"/>
+    <s v="NN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="2"/>
+  </r>
+  <r>
+    <d v="2015-02-15T00:00:00"/>
+    <n v="235"/>
+    <s v="EN"/>
+    <n v="0"/>
+    <s v="l2"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <d v="2015-02-15T00:00:00"/>
+    <n v="235"/>
+    <s v="EN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <d v="2015-02-15T00:00:00"/>
+    <n v="235"/>
+    <s v="SVR"/>
+    <n v="8"/>
+    <s v="l1"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <d v="2015-02-15T00:00:00"/>
+    <n v="235"/>
+    <s v="NN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <d v="2015-02-15T00:00:00"/>
+    <n v="252.4"/>
+    <s v="EN"/>
+    <n v="0"/>
+    <s v="l2"/>
+    <x v="6"/>
+  </r>
+  <r>
+    <d v="2015-02-15T00:00:00"/>
+    <n v="212.7"/>
+    <s v="EN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="3"/>
+  </r>
+  <r>
+    <d v="2015-02-15T00:00:00"/>
+    <n v="222.9"/>
+    <s v="SVR"/>
+    <n v="8"/>
+    <s v="l1"/>
+    <x v="2"/>
+  </r>
+  <r>
+    <d v="2015-02-15T00:00:00"/>
+    <n v="212.7"/>
+    <s v="NN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="3"/>
+  </r>
+  <r>
+    <d v="2015-02-16T00:00:00"/>
+    <n v="183.9"/>
+    <s v="EN"/>
+    <n v="0"/>
+    <s v="l2"/>
+    <x v="10"/>
+  </r>
+  <r>
+    <d v="2015-02-16T00:00:00"/>
+    <n v="213.2"/>
+    <s v="EN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="3"/>
+  </r>
+  <r>
+    <d v="2015-02-16T00:00:00"/>
+    <n v="177.7"/>
+    <s v="SVR"/>
+    <n v="8"/>
+    <s v="l1"/>
+    <x v="10"/>
+  </r>
+  <r>
+    <d v="2015-02-16T00:00:00"/>
+    <n v="190.8"/>
+    <s v="NN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="7"/>
+  </r>
+  <r>
+    <d v="2015-02-17T00:00:00"/>
+    <n v="150.69999999999999"/>
+    <s v="EN"/>
+    <n v="0"/>
+    <s v="l2"/>
+    <x v="13"/>
+  </r>
+  <r>
+    <d v="2015-02-17T00:00:00"/>
+    <n v="176.9"/>
+    <s v="EN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="10"/>
+  </r>
+  <r>
+    <d v="2015-02-17T00:00:00"/>
+    <n v="150.5"/>
+    <s v="SVR"/>
+    <n v="8"/>
+    <s v="l1"/>
+    <x v="13"/>
+  </r>
+  <r>
+    <d v="2015-02-17T00:00:00"/>
+    <n v="191"/>
+    <s v="NN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="7"/>
+  </r>
+  <r>
+    <d v="2015-02-18T00:00:00"/>
+    <n v="235.5"/>
+    <s v="EN"/>
+    <n v="0"/>
+    <s v="l2"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <d v="2015-02-18T00:00:00"/>
+    <n v="226.9"/>
+    <s v="EN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="5"/>
+  </r>
+  <r>
+    <d v="2015-02-18T00:00:00"/>
+    <n v="226.9"/>
+    <s v="SVR"/>
+    <n v="8"/>
+    <s v="l1"/>
+    <x v="5"/>
+  </r>
+  <r>
+    <d v="2015-02-18T00:00:00"/>
+    <n v="226.9"/>
+    <s v="NN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="5"/>
+  </r>
+  <r>
+    <d v="2015-02-19T00:00:00"/>
+    <n v="176.1"/>
+    <s v="EN"/>
+    <n v="0"/>
+    <s v="l2"/>
+    <x v="10"/>
+  </r>
+  <r>
+    <d v="2015-02-19T00:00:00"/>
+    <n v="219.4"/>
+    <s v="EN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="2"/>
+  </r>
+  <r>
+    <d v="2015-02-19T00:00:00"/>
+    <n v="197.2"/>
+    <s v="SVR"/>
+    <n v="8"/>
+    <s v="l1"/>
+    <x v="12"/>
+  </r>
+  <r>
+    <d v="2015-02-19T00:00:00"/>
+    <n v="221"/>
+    <s v="NN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="2"/>
+  </r>
+  <r>
+    <d v="2015-02-20T00:00:00"/>
+    <n v="211.3"/>
+    <s v="EN"/>
+    <n v="0"/>
+    <s v="l2"/>
+    <x v="3"/>
+  </r>
+  <r>
+    <d v="2015-02-20T00:00:00"/>
+    <n v="269"/>
+    <s v="EN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="11"/>
+  </r>
+  <r>
+    <d v="2015-02-20T00:00:00"/>
+    <n v="228"/>
+    <s v="SVR"/>
+    <n v="8"/>
+    <s v="l1"/>
+    <x v="5"/>
+  </r>
+  <r>
+    <d v="2015-02-20T00:00:00"/>
+    <n v="250.8"/>
+    <s v="NN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="6"/>
+  </r>
+  <r>
+    <d v="2015-02-20T00:00:00"/>
+    <n v="168.3"/>
+    <s v="EN"/>
+    <n v="0"/>
+    <s v="l2"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <d v="2015-02-20T00:00:00"/>
+    <n v="152.80000000000001"/>
+    <s v="EN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="13"/>
+  </r>
+  <r>
+    <d v="2015-02-20T00:00:00"/>
+    <n v="158.1"/>
+    <s v="SVR"/>
+    <n v="8"/>
+    <s v="l1"/>
+    <x v="9"/>
+  </r>
+  <r>
+    <d v="2015-02-20T00:00:00"/>
+    <n v="175.8"/>
+    <s v="NN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="10"/>
+  </r>
+  <r>
+    <d v="2015-02-21T00:00:00"/>
+    <n v="216.5"/>
+    <s v="EN"/>
+    <n v="0"/>
+    <s v="l2"/>
+    <x v="2"/>
+  </r>
+  <r>
+    <d v="2015-02-21T00:00:00"/>
+    <n v="216.5"/>
+    <s v="EN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="2"/>
+  </r>
+  <r>
+    <d v="2015-02-21T00:00:00"/>
+    <n v="238.3"/>
+    <s v="SVR"/>
+    <n v="8"/>
+    <s v="l1"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <d v="2015-02-21T00:00:00"/>
+    <n v="256.7"/>
+    <s v="NN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="4"/>
+  </r>
+  <r>
+    <d v="2015-02-21T00:00:00"/>
+    <n v="231.9"/>
+    <s v="EN"/>
+    <n v="0"/>
+    <s v="l2"/>
+    <x v="5"/>
+  </r>
+  <r>
+    <d v="2015-02-21T00:00:00"/>
+    <n v="231.9"/>
+    <s v="EN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="5"/>
+  </r>
+  <r>
+    <d v="2015-02-21T00:00:00"/>
+    <n v="208.9"/>
+    <s v="SVR"/>
+    <n v="8"/>
+    <s v="l1"/>
+    <x v="3"/>
+  </r>
+  <r>
+    <d v="2015-02-21T00:00:00"/>
+    <n v="231.9"/>
+    <s v="NN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="5"/>
+  </r>
+  <r>
+    <d v="2015-02-22T00:00:00"/>
+    <n v="207.9"/>
+    <s v="EN"/>
+    <n v="0"/>
+    <s v="l2"/>
+    <x v="3"/>
+  </r>
+  <r>
+    <d v="2015-02-22T00:00:00"/>
+    <n v="188.7"/>
+    <s v="EN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="7"/>
+  </r>
+  <r>
+    <d v="2015-02-22T00:00:00"/>
+    <n v="205.3"/>
+    <s v="SVR"/>
+    <n v="8"/>
+    <s v="l1"/>
+    <x v="3"/>
+  </r>
+  <r>
+    <d v="2015-02-22T00:00:00"/>
+    <n v="189"/>
+    <s v="NN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="7"/>
+  </r>
+  <r>
+    <d v="2015-02-23T00:00:00"/>
+    <n v="200.7"/>
+    <s v="EN"/>
+    <n v="0"/>
+    <s v="l2"/>
+    <x v="12"/>
+  </r>
+  <r>
+    <d v="2015-02-23T00:00:00"/>
+    <n v="200.7"/>
+    <s v="EN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="12"/>
+  </r>
+  <r>
+    <d v="2015-02-23T00:00:00"/>
+    <n v="158.1"/>
+    <s v="SVR"/>
+    <n v="8"/>
+    <s v="l1"/>
+    <x v="9"/>
+  </r>
+  <r>
+    <d v="2015-02-23T00:00:00"/>
+    <n v="212.7"/>
+    <s v="NN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="3"/>
+  </r>
+  <r>
+    <d v="2015-02-24T00:00:00"/>
+    <n v="218.3"/>
+    <s v="EN"/>
+    <n v="0"/>
+    <s v="l2"/>
+    <x v="2"/>
+  </r>
+  <r>
+    <d v="2015-02-24T00:00:00"/>
+    <n v="231.9"/>
+    <s v="EN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="5"/>
+  </r>
+  <r>
+    <d v="2015-02-24T00:00:00"/>
+    <n v="246.3"/>
+    <s v="SVR"/>
+    <n v="8"/>
+    <s v="l1"/>
+    <x v="6"/>
+  </r>
+  <r>
+    <d v="2015-02-24T00:00:00"/>
+    <n v="218.5"/>
+    <s v="NN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="2"/>
+  </r>
+  <r>
+    <d v="2015-02-25T00:00:00"/>
+    <n v="221"/>
+    <s v="EN"/>
+    <n v="0"/>
+    <s v="l2"/>
+    <x v="2"/>
+  </r>
+  <r>
+    <d v="2015-02-25T00:00:00"/>
+    <n v="188"/>
+    <s v="EN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="7"/>
+  </r>
+  <r>
+    <d v="2015-02-25T00:00:00"/>
+    <n v="209.1"/>
+    <s v="SVR"/>
+    <n v="8"/>
+    <s v="l1"/>
+    <x v="3"/>
+  </r>
+  <r>
+    <d v="2015-02-25T00:00:00"/>
+    <n v="192"/>
+    <s v="NN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="7"/>
+  </r>
+  <r>
+    <d v="2015-02-27T00:00:00"/>
+    <n v="171.4"/>
+    <s v="EN"/>
+    <n v="0"/>
+    <s v="l2"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <d v="2015-02-27T00:00:00"/>
+    <n v="171.4"/>
+    <s v="EN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <d v="2015-02-27T00:00:00"/>
+    <n v="174.2"/>
+    <s v="SVR"/>
+    <n v="8"/>
+    <s v="l1"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <d v="2015-02-27T00:00:00"/>
+    <n v="184.7"/>
+    <s v="NN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="10"/>
+  </r>
+  <r>
+    <d v="2015-02-28T00:00:00"/>
+    <n v="228.1"/>
+    <s v="EN"/>
+    <n v="0"/>
+    <s v="l2"/>
+    <x v="5"/>
+  </r>
+  <r>
+    <d v="2015-02-28T00:00:00"/>
+    <n v="206.5"/>
+    <s v="EN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="3"/>
+  </r>
+  <r>
+    <d v="2015-02-28T00:00:00"/>
+    <n v="221.9"/>
+    <s v="SVR"/>
+    <n v="8"/>
+    <s v="l1"/>
+    <x v="2"/>
+  </r>
+  <r>
+    <d v="2015-02-28T00:00:00"/>
+    <n v="221.9"/>
+    <s v="NN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="2"/>
+  </r>
+  <r>
+    <d v="2015-03-01T00:00:00"/>
+    <n v="235.7"/>
+    <s v="EN"/>
+    <n v="0"/>
+    <s v="l2"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <d v="2015-03-01T00:00:00"/>
+    <n v="205.8"/>
+    <s v="EN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="3"/>
+  </r>
+  <r>
+    <d v="2015-03-01T00:00:00"/>
+    <n v="257.2"/>
+    <s v="SVR"/>
+    <n v="8"/>
+    <s v="l1"/>
+    <x v="4"/>
+  </r>
+  <r>
+    <d v="2015-03-01T00:00:00"/>
+    <n v="206"/>
+    <s v="NN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="3"/>
+  </r>
+  <r>
+    <d v="2015-03-01T00:00:00"/>
+    <n v="202.2"/>
+    <s v="EN"/>
+    <n v="0"/>
+    <s v="l2"/>
+    <x v="12"/>
+  </r>
+  <r>
+    <d v="2015-03-01T00:00:00"/>
+    <n v="202.2"/>
+    <s v="EN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="12"/>
+  </r>
+  <r>
+    <d v="2015-03-01T00:00:00"/>
+    <n v="185.9"/>
+    <s v="SVR"/>
+    <n v="8"/>
+    <s v="l1"/>
+    <x v="7"/>
+  </r>
+  <r>
+    <d v="2015-03-01T00:00:00"/>
+    <n v="202.2"/>
+    <s v="NN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="12"/>
+  </r>
+  <r>
+    <d v="2015-03-02T00:00:00"/>
+    <n v="202.1"/>
+    <s v="EN"/>
+    <n v="0"/>
+    <s v="l2"/>
+    <x v="12"/>
+  </r>
+  <r>
+    <d v="2015-03-02T00:00:00"/>
+    <n v="202.1"/>
+    <s v="EN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="12"/>
+  </r>
+  <r>
+    <d v="2015-03-02T00:00:00"/>
+    <n v="197.4"/>
+    <s v="SVR"/>
+    <n v="8"/>
+    <s v="l1"/>
+    <x v="12"/>
+  </r>
+  <r>
+    <d v="2015-03-02T00:00:00"/>
+    <n v="202.1"/>
+    <s v="NN"/>
+    <n v="8"/>
+    <s v="l2"/>
+    <x v="12"/>
   </r>
 </pivotCacheRecords>
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable1" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="4" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="4" indent="0" outline="1" outlineData="1" gridDropZones="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable1" cacheId="61" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="4" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="4" indent="0" outline="1" outlineData="1" gridDropZones="1" multipleFieldFilters="0">
   <location ref="A3:B20" firstHeaderRow="2" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="6">
     <pivotField numFmtId="14" showAll="0"/>
@@ -2773,26 +3884,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="53" customHeight="1">
-      <c r="B1" s="23" t="s">
+      <c r="B1" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23" t="s">
+      <c r="C1" s="24"/>
+      <c r="D1" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23" t="s">
+      <c r="E1" s="24"/>
+      <c r="F1" s="24" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="23"/>
-      <c r="H1" s="23" t="s">
+      <c r="G1" s="24"/>
+      <c r="H1" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="23"/>
-      <c r="J1" s="23" t="s">
+      <c r="I1" s="24"/>
+      <c r="J1" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="K1" s="23"/>
+      <c r="K1" s="24"/>
     </row>
     <row r="2" spans="1:12" ht="15" customHeight="1">
       <c r="A2" t="s">
@@ -3497,7 +4608,7 @@
       </c>
       <c r="W3">
         <f>_xlfn.NORM.DIST(V3,Sheet4!$J$2,Sheet4!$J$3,FALSE)</f>
-        <v>1.1393633168699394E-3</v>
+        <v>1.2322576564640026E-3</v>
       </c>
     </row>
     <row r="4" spans="1:23">
@@ -3512,7 +4623,7 @@
       </c>
       <c r="W4">
         <f>_xlfn.NORM.DIST(V4,Sheet4!$J$2,Sheet4!$J$3,FALSE)</f>
-        <v>2.2390141961175767E-3</v>
+        <v>2.4771783512800303E-3</v>
       </c>
     </row>
     <row r="5" spans="1:23">
@@ -3520,14 +4631,14 @@
         <v>150</v>
       </c>
       <c r="B5" s="18">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="V5">
         <v>170</v>
       </c>
       <c r="W5">
         <f>_xlfn.NORM.DIST(V5,Sheet4!$J$2,Sheet4!$J$3,FALSE)</f>
-        <v>3.9460392509322595E-3</v>
+        <v>4.4211965360106409E-3</v>
       </c>
     </row>
     <row r="6" spans="1:23">
@@ -3535,14 +4646,14 @@
         <v>160</v>
       </c>
       <c r="B6" s="18">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="V6">
         <v>180</v>
       </c>
       <c r="W6">
         <f>_xlfn.NORM.DIST(V6,Sheet4!$J$2,Sheet4!$J$3,FALSE)</f>
-        <v>6.2370021495231475E-3</v>
+        <v>7.0056616851002533E-3</v>
       </c>
     </row>
     <row r="7" spans="1:23">
@@ -3550,14 +4661,14 @@
         <v>170</v>
       </c>
       <c r="B7" s="18">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="V7">
         <v>190</v>
       </c>
       <c r="W7">
         <f>_xlfn.NORM.DIST(V7,Sheet4!$J$2,Sheet4!$J$3,FALSE)</f>
-        <v>8.8409783254578614E-3</v>
+        <v>9.8556505132881399E-3</v>
       </c>
     </row>
     <row r="8" spans="1:23">
@@ -3565,14 +4676,14 @@
         <v>180</v>
       </c>
       <c r="B8" s="18">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="V8">
         <v>200</v>
       </c>
       <c r="W8">
         <f>_xlfn.NORM.DIST(V8,Sheet4!$J$2,Sheet4!$J$3,FALSE)</f>
-        <v>1.1239181825555446E-2</v>
+        <v>1.2309721384704569E-2</v>
       </c>
     </row>
     <row r="9" spans="1:23">
@@ -3580,14 +4691,14 @@
         <v>190</v>
       </c>
       <c r="B9" s="18">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="V9">
         <v>210</v>
       </c>
       <c r="W9">
         <f>_xlfn.NORM.DIST(V9,Sheet4!$J$2,Sheet4!$J$3,FALSE)</f>
-        <v>1.2813831471045038E-2</v>
+        <v>1.3650166423317553E-2</v>
       </c>
     </row>
     <row r="10" spans="1:23">
@@ -3595,14 +4706,14 @@
         <v>200</v>
       </c>
       <c r="B10" s="18">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="V10">
         <v>220</v>
       </c>
       <c r="W10">
         <f>_xlfn.NORM.DIST(V10,Sheet4!$J$2,Sheet4!$J$3,FALSE)</f>
-        <v>1.3101869145774273E-2</v>
+        <v>1.3438613506130237E-2</v>
       </c>
     </row>
     <row r="11" spans="1:23">
@@ -3610,14 +4721,14 @@
         <v>210</v>
       </c>
       <c r="B11" s="18">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="V11">
         <v>230</v>
       </c>
       <c r="W11">
         <f>_xlfn.NORM.DIST(V11,Sheet4!$J$2,Sheet4!$J$3,FALSE)</f>
-        <v>1.2014271630391963E-2</v>
+        <v>1.1746210401513217E-2</v>
       </c>
     </row>
     <row r="12" spans="1:23">
@@ -3625,14 +4736,14 @@
         <v>220</v>
       </c>
       <c r="B12" s="18">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="V12">
         <v>240</v>
       </c>
       <c r="W12">
         <f>_xlfn.NORM.DIST(V12,Sheet4!$J$2,Sheet4!$J$3,FALSE)</f>
-        <v>9.8803328398412143E-3</v>
+        <v>9.1152352628045517E-3</v>
       </c>
     </row>
     <row r="13" spans="1:23">
@@ -3640,14 +4751,14 @@
         <v>230</v>
       </c>
       <c r="B13" s="18">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="V13">
         <v>250</v>
       </c>
       <c r="W13">
         <f>_xlfn.NORM.DIST(V13,Sheet4!$J$2,Sheet4!$J$3,FALSE)</f>
-        <v>7.2871153216842394E-3</v>
+        <v>6.2800743168478241E-3</v>
       </c>
     </row>
     <row r="14" spans="1:23">
@@ -3655,14 +4766,14 @@
         <v>240</v>
       </c>
       <c r="B14" s="18">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="V14">
         <v>260</v>
       </c>
       <c r="W14">
         <f>_xlfn.NORM.DIST(V14,Sheet4!$J$2,Sheet4!$J$3,FALSE)</f>
-        <v>4.8200289779360391E-3</v>
+        <v>3.8413906809498812E-3</v>
       </c>
     </row>
     <row r="15" spans="1:23">
@@ -3670,14 +4781,14 @@
         <v>250</v>
       </c>
       <c r="B15" s="18">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="V15">
         <v>270</v>
       </c>
       <c r="W15">
         <f>_xlfn.NORM.DIST(V15,Sheet4!$J$2,Sheet4!$J$3,FALSE)</f>
-        <v>2.8592596478103334E-3</v>
+        <v>2.0861184702722761E-3</v>
       </c>
     </row>
     <row r="16" spans="1:23">
@@ -3685,14 +4796,14 @@
         <v>260</v>
       </c>
       <c r="B16" s="18">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="V16">
         <v>280</v>
       </c>
       <c r="W16">
         <f>_xlfn.NORM.DIST(V16,Sheet4!$J$2,Sheet4!$J$3,FALSE)</f>
-        <v>1.5211340235296864E-3</v>
+        <v>1.0058107027238546E-3</v>
       </c>
     </row>
     <row r="17" spans="1:23">
@@ -3700,14 +4811,14 @@
         <v>270</v>
       </c>
       <c r="B17" s="18">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="V17">
         <v>290</v>
       </c>
       <c r="W17">
         <f>_xlfn.NORM.DIST(V17,Sheet4!$J$2,Sheet4!$J$3,FALSE)</f>
-        <v>7.2575711948566013E-4</v>
+        <v>4.3054676592934135E-4</v>
       </c>
     </row>
     <row r="18" spans="1:23">
@@ -3731,7 +4842,7 @@
         <v>10</v>
       </c>
       <c r="B20" s="18">
-        <v>147</v>
+        <v>235</v>
       </c>
     </row>
   </sheetData>
@@ -3747,8 +4858,8 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J200"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0"/>
+  <dimension ref="A1:J1048576"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.75"/>
   <cols>
     <col min="7" max="7" width="24.6640625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="12.1640625" bestFit="1" customWidth="1"/>
@@ -3802,7 +4913,7 @@
       </c>
       <c r="J2">
         <f>AVERAGE(B:B)</f>
-        <v>217.04149659863958</v>
+        <v>213.68723404255331</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="18">
@@ -3830,7 +4941,7 @@
       </c>
       <c r="J3">
         <f>_xlfn.STDEV.S(B:B)</f>
-        <v>30.304506748198964</v>
+        <v>28.99075019756452</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="18">
@@ -6370,7 +7481,7 @@
         <v>19</v>
       </c>
       <c r="F106">
-        <f t="shared" ref="F106:F148" si="4">ROUND(B106/10,0)*10</f>
+        <f t="shared" ref="F106:F169" si="4">ROUND(B106/10,0)*10</f>
         <v>290</v>
       </c>
       <c r="G106" s="22" t="s">
@@ -7518,6 +8629,9 @@
       <c r="A149" s="1">
         <v>42047</v>
       </c>
+      <c r="B149">
+        <v>216.5</v>
+      </c>
       <c r="C149" s="20" t="s">
         <v>12</v>
       </c>
@@ -7526,6 +8640,10 @@
       </c>
       <c r="E149" s="19" t="s">
         <v>13</v>
+      </c>
+      <c r="F149">
+        <f t="shared" si="4"/>
+        <v>220</v>
       </c>
       <c r="G149" s="22" t="s">
         <v>72</v>
@@ -7538,6 +8656,9 @@
       <c r="A150" s="1">
         <v>42047</v>
       </c>
+      <c r="B150">
+        <v>216.5</v>
+      </c>
       <c r="C150" s="20" t="s">
         <v>12</v>
       </c>
@@ -7546,6 +8667,10 @@
       </c>
       <c r="E150" s="19" t="s">
         <v>13</v>
+      </c>
+      <c r="F150">
+        <f t="shared" si="4"/>
+        <v>220</v>
       </c>
       <c r="G150" s="22" t="s">
         <v>72</v>
@@ -7558,6 +8683,9 @@
       <c r="A151" s="1">
         <v>42047</v>
       </c>
+      <c r="B151">
+        <v>166.3</v>
+      </c>
       <c r="C151" s="20" t="s">
         <v>20</v>
       </c>
@@ -7566,6 +8694,10 @@
       </c>
       <c r="E151" s="19" t="s">
         <v>19</v>
+      </c>
+      <c r="F151">
+        <f t="shared" si="4"/>
+        <v>170</v>
       </c>
       <c r="G151" s="22" t="s">
         <v>71</v>
@@ -7578,6 +8710,9 @@
       <c r="A152" s="1">
         <v>42047</v>
       </c>
+      <c r="B152">
+        <v>168</v>
+      </c>
       <c r="C152" s="20" t="s">
         <v>56</v>
       </c>
@@ -7587,6 +8722,10 @@
       <c r="E152" s="19" t="s">
         <v>13</v>
       </c>
+      <c r="F152">
+        <f t="shared" si="4"/>
+        <v>170</v>
+      </c>
       <c r="G152" s="22" t="s">
         <v>70</v>
       </c>
@@ -7594,247 +8733,2311 @@
         <v>0</v>
       </c>
     </row>
-    <row r="153" spans="1:9">
+    <row r="153" spans="1:9" ht="25">
+      <c r="A153" s="1">
+        <v>42049</v>
+      </c>
+      <c r="B153">
+        <v>195.1</v>
+      </c>
+      <c r="C153" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D153" s="20">
+        <v>0</v>
+      </c>
+      <c r="E153" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F153">
+        <f t="shared" si="4"/>
+        <v>200</v>
+      </c>
+      <c r="G153" s="22" t="s">
+        <v>73</v>
+      </c>
       <c r="I153">
         <v>0</v>
       </c>
     </row>
-    <row r="154" spans="1:9">
+    <row r="154" spans="1:9" ht="25">
+      <c r="A154" s="1">
+        <v>42049</v>
+      </c>
+      <c r="B154">
+        <v>222.4</v>
+      </c>
+      <c r="C154" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D154" s="20">
+        <v>8</v>
+      </c>
+      <c r="E154" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F154">
+        <f t="shared" si="4"/>
+        <v>220</v>
+      </c>
+      <c r="G154" s="22" t="s">
+        <v>74</v>
+      </c>
       <c r="I154">
         <v>0</v>
       </c>
     </row>
-    <row r="155" spans="1:9">
+    <row r="155" spans="1:9" ht="25">
+      <c r="A155" s="1">
+        <v>42049</v>
+      </c>
+      <c r="B155">
+        <v>205</v>
+      </c>
+      <c r="C155" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="D155" s="20">
+        <v>8</v>
+      </c>
+      <c r="E155" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F155">
+        <f t="shared" si="4"/>
+        <v>210</v>
+      </c>
+      <c r="G155" s="22" t="s">
+        <v>75</v>
+      </c>
       <c r="I155">
         <v>0</v>
       </c>
     </row>
-    <row r="156" spans="1:9">
+    <row r="156" spans="1:9" ht="25">
+      <c r="A156" s="1">
+        <v>42049</v>
+      </c>
+      <c r="B156">
+        <v>222.4</v>
+      </c>
+      <c r="C156" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="D156" s="20">
+        <v>8</v>
+      </c>
+      <c r="E156" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F156">
+        <f t="shared" si="4"/>
+        <v>220</v>
+      </c>
+      <c r="G156" s="22" t="s">
+        <v>74</v>
+      </c>
       <c r="I156">
         <v>0</v>
       </c>
     </row>
-    <row r="157" spans="1:9">
+    <row r="157" spans="1:9" ht="25">
+      <c r="A157" s="1">
+        <v>42049</v>
+      </c>
+      <c r="B157">
+        <v>200</v>
+      </c>
+      <c r="C157" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D157" s="20">
+        <v>0</v>
+      </c>
+      <c r="E157" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F157">
+        <f t="shared" si="4"/>
+        <v>200</v>
+      </c>
+      <c r="G157" s="22" t="s">
+        <v>76</v>
+      </c>
       <c r="I157">
         <v>0</v>
       </c>
     </row>
-    <row r="158" spans="1:9">
+    <row r="158" spans="1:9" ht="25">
+      <c r="A158" s="1">
+        <v>42049</v>
+      </c>
+      <c r="B158">
+        <v>234.8</v>
+      </c>
+      <c r="C158" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D158" s="20">
+        <v>8</v>
+      </c>
+      <c r="E158" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F158">
+        <f t="shared" si="4"/>
+        <v>230</v>
+      </c>
+      <c r="G158" s="22" t="s">
+        <v>77</v>
+      </c>
       <c r="I158">
         <v>0</v>
       </c>
     </row>
-    <row r="159" spans="1:9">
+    <row r="159" spans="1:9" ht="25">
+      <c r="A159" s="1">
+        <v>42049</v>
+      </c>
+      <c r="B159">
+        <v>222.3</v>
+      </c>
+      <c r="C159" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="D159" s="20">
+        <v>8</v>
+      </c>
+      <c r="E159" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F159">
+        <f t="shared" si="4"/>
+        <v>220</v>
+      </c>
+      <c r="G159" s="22" t="s">
+        <v>78</v>
+      </c>
       <c r="I159">
         <v>0</v>
       </c>
     </row>
-    <row r="160" spans="1:9">
+    <row r="160" spans="1:9" ht="25">
+      <c r="A160" s="1">
+        <v>42049</v>
+      </c>
+      <c r="B160">
+        <v>220.9</v>
+      </c>
+      <c r="C160" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="D160" s="20">
+        <v>8</v>
+      </c>
+      <c r="E160" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F160">
+        <f t="shared" si="4"/>
+        <v>220</v>
+      </c>
+      <c r="G160" s="22" t="s">
+        <v>79</v>
+      </c>
       <c r="I160">
         <v>0</v>
       </c>
     </row>
-    <row r="161" spans="9:9">
+    <row r="161" spans="1:9" ht="25">
+      <c r="A161" s="1">
+        <v>42050</v>
+      </c>
+      <c r="B161">
+        <v>235</v>
+      </c>
+      <c r="C161" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D161" s="20">
+        <v>0</v>
+      </c>
+      <c r="E161" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F161">
+        <f t="shared" si="4"/>
+        <v>240</v>
+      </c>
+      <c r="G161" s="22" t="s">
+        <v>80</v>
+      </c>
       <c r="I161">
         <v>0</v>
       </c>
     </row>
-    <row r="162" spans="9:9">
+    <row r="162" spans="1:9" ht="25">
+      <c r="A162" s="1">
+        <v>42050</v>
+      </c>
+      <c r="B162">
+        <v>235</v>
+      </c>
+      <c r="C162" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D162" s="20">
+        <v>8</v>
+      </c>
+      <c r="E162" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F162">
+        <f t="shared" si="4"/>
+        <v>240</v>
+      </c>
+      <c r="G162" s="22" t="s">
+        <v>80</v>
+      </c>
       <c r="I162">
         <v>0</v>
       </c>
     </row>
-    <row r="163" spans="9:9">
+    <row r="163" spans="1:9" ht="25">
+      <c r="A163" s="1">
+        <v>42050</v>
+      </c>
+      <c r="B163">
+        <v>235</v>
+      </c>
+      <c r="C163" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="D163" s="20">
+        <v>8</v>
+      </c>
+      <c r="E163" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F163">
+        <f t="shared" si="4"/>
+        <v>240</v>
+      </c>
+      <c r="G163" s="22" t="s">
+        <v>80</v>
+      </c>
       <c r="I163">
         <v>0</v>
       </c>
     </row>
-    <row r="164" spans="9:9">
+    <row r="164" spans="1:9" ht="25">
+      <c r="A164" s="1">
+        <v>42050</v>
+      </c>
+      <c r="B164">
+        <v>235</v>
+      </c>
+      <c r="C164" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="D164" s="20">
+        <v>8</v>
+      </c>
+      <c r="E164" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F164">
+        <f t="shared" si="4"/>
+        <v>240</v>
+      </c>
+      <c r="G164" s="22" t="s">
+        <v>80</v>
+      </c>
       <c r="I164">
         <v>0</v>
       </c>
     </row>
-    <row r="165" spans="9:9">
+    <row r="165" spans="1:9" ht="25">
+      <c r="A165" s="1">
+        <v>42050</v>
+      </c>
+      <c r="B165">
+        <v>252.4</v>
+      </c>
+      <c r="C165" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D165" s="20">
+        <v>0</v>
+      </c>
+      <c r="E165" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F165">
+        <f t="shared" si="4"/>
+        <v>250</v>
+      </c>
+      <c r="G165" s="22" t="s">
+        <v>82</v>
+      </c>
       <c r="I165">
         <v>0</v>
       </c>
     </row>
-    <row r="166" spans="9:9">
+    <row r="166" spans="1:9" ht="25">
+      <c r="A166" s="1">
+        <v>42050</v>
+      </c>
+      <c r="B166">
+        <v>212.7</v>
+      </c>
+      <c r="C166" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D166" s="20">
+        <v>8</v>
+      </c>
+      <c r="E166" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F166">
+        <f t="shared" si="4"/>
+        <v>210</v>
+      </c>
+      <c r="G166" s="22" t="s">
+        <v>81</v>
+      </c>
       <c r="I166">
         <v>0</v>
       </c>
     </row>
-    <row r="167" spans="9:9">
+    <row r="167" spans="1:9" ht="25">
+      <c r="A167" s="1">
+        <v>42050</v>
+      </c>
+      <c r="B167">
+        <v>222.9</v>
+      </c>
+      <c r="C167" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="D167" s="20">
+        <v>8</v>
+      </c>
+      <c r="E167" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F167">
+        <f t="shared" si="4"/>
+        <v>220</v>
+      </c>
+      <c r="G167" s="22" t="s">
+        <v>83</v>
+      </c>
       <c r="I167">
         <v>0</v>
       </c>
     </row>
-    <row r="168" spans="9:9">
+    <row r="168" spans="1:9" ht="25">
+      <c r="A168" s="1">
+        <v>42050</v>
+      </c>
+      <c r="B168">
+        <v>212.7</v>
+      </c>
+      <c r="C168" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="D168" s="20">
+        <v>8</v>
+      </c>
+      <c r="E168" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F168">
+        <f t="shared" si="4"/>
+        <v>210</v>
+      </c>
+      <c r="G168" s="22" t="s">
+        <v>81</v>
+      </c>
       <c r="I168">
         <v>0</v>
       </c>
     </row>
-    <row r="169" spans="9:9">
+    <row r="169" spans="1:9" ht="25">
+      <c r="A169" s="1">
+        <v>42051</v>
+      </c>
+      <c r="B169">
+        <v>183.9</v>
+      </c>
+      <c r="C169" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D169" s="20">
+        <v>0</v>
+      </c>
+      <c r="E169" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F169">
+        <f t="shared" si="4"/>
+        <v>180</v>
+      </c>
+      <c r="G169" s="22" t="s">
+        <v>84</v>
+      </c>
       <c r="I169">
         <v>0</v>
       </c>
     </row>
-    <row r="170" spans="9:9">
+    <row r="170" spans="1:9" ht="25">
+      <c r="A170" s="1">
+        <v>42051</v>
+      </c>
+      <c r="B170">
+        <v>213.2</v>
+      </c>
+      <c r="C170" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D170" s="20">
+        <v>8</v>
+      </c>
+      <c r="E170" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F170">
+        <f t="shared" ref="F170:F233" si="5">ROUND(B170/10,0)*10</f>
+        <v>210</v>
+      </c>
+      <c r="G170" s="22" t="s">
+        <v>85</v>
+      </c>
       <c r="I170">
         <v>0</v>
       </c>
     </row>
-    <row r="171" spans="9:9">
+    <row r="171" spans="1:9" ht="25">
+      <c r="A171" s="1">
+        <v>42051</v>
+      </c>
+      <c r="B171">
+        <v>177.7</v>
+      </c>
+      <c r="C171" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="D171" s="20">
+        <v>8</v>
+      </c>
+      <c r="E171" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F171">
+        <f t="shared" si="5"/>
+        <v>180</v>
+      </c>
+      <c r="G171" s="22" t="s">
+        <v>86</v>
+      </c>
       <c r="I171">
         <v>0</v>
       </c>
     </row>
-    <row r="172" spans="9:9">
+    <row r="172" spans="1:9" ht="25">
+      <c r="A172" s="1">
+        <v>42051</v>
+      </c>
+      <c r="B172">
+        <v>190.8</v>
+      </c>
+      <c r="C172" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="D172" s="20">
+        <v>8</v>
+      </c>
+      <c r="E172" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F172">
+        <f t="shared" si="5"/>
+        <v>190</v>
+      </c>
+      <c r="G172" s="22" t="s">
+        <v>87</v>
+      </c>
       <c r="I172">
         <v>0</v>
       </c>
     </row>
-    <row r="173" spans="9:9">
+    <row r="173" spans="1:9" ht="25">
+      <c r="A173" s="1">
+        <v>42052</v>
+      </c>
+      <c r="B173">
+        <v>150.69999999999999</v>
+      </c>
+      <c r="C173" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D173" s="20">
+        <v>0</v>
+      </c>
+      <c r="E173" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F173">
+        <f t="shared" si="5"/>
+        <v>150</v>
+      </c>
+      <c r="G173" s="22" t="s">
+        <v>88</v>
+      </c>
       <c r="I173">
         <v>0</v>
       </c>
     </row>
-    <row r="174" spans="9:9">
+    <row r="174" spans="1:9" ht="25">
+      <c r="A174" s="1">
+        <v>42052</v>
+      </c>
+      <c r="B174">
+        <v>176.9</v>
+      </c>
+      <c r="C174" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D174" s="20">
+        <v>8</v>
+      </c>
+      <c r="E174" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F174">
+        <f t="shared" si="5"/>
+        <v>180</v>
+      </c>
+      <c r="G174" s="22" t="s">
+        <v>89</v>
+      </c>
       <c r="I174">
         <v>0</v>
       </c>
     </row>
-    <row r="175" spans="9:9">
+    <row r="175" spans="1:9" ht="25">
+      <c r="A175" s="1">
+        <v>42052</v>
+      </c>
+      <c r="B175">
+        <v>150.5</v>
+      </c>
+      <c r="C175" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="D175" s="20">
+        <v>8</v>
+      </c>
+      <c r="E175" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F175">
+        <f t="shared" si="5"/>
+        <v>150</v>
+      </c>
+      <c r="G175" s="22" t="s">
+        <v>90</v>
+      </c>
       <c r="I175">
         <v>0</v>
       </c>
     </row>
-    <row r="176" spans="9:9">
+    <row r="176" spans="1:9" ht="25">
+      <c r="A176" s="1">
+        <v>42052</v>
+      </c>
+      <c r="B176">
+        <v>191</v>
+      </c>
+      <c r="C176" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="D176" s="20">
+        <v>8</v>
+      </c>
+      <c r="E176" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F176">
+        <f t="shared" si="5"/>
+        <v>190</v>
+      </c>
+      <c r="G176" s="22" t="s">
+        <v>91</v>
+      </c>
       <c r="I176">
         <v>0</v>
       </c>
     </row>
-    <row r="177" spans="9:9">
+    <row r="177" spans="1:9" ht="25">
+      <c r="A177" s="1">
+        <v>42053</v>
+      </c>
+      <c r="B177">
+        <v>235.5</v>
+      </c>
+      <c r="C177" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D177" s="20">
+        <v>0</v>
+      </c>
+      <c r="E177" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F177">
+        <f t="shared" si="5"/>
+        <v>240</v>
+      </c>
+      <c r="G177" s="22" t="s">
+        <v>92</v>
+      </c>
       <c r="I177">
         <v>0</v>
       </c>
     </row>
-    <row r="178" spans="9:9">
+    <row r="178" spans="1:9" ht="25">
+      <c r="A178" s="1">
+        <v>42053</v>
+      </c>
+      <c r="B178">
+        <v>226.9</v>
+      </c>
+      <c r="C178" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D178" s="20">
+        <v>8</v>
+      </c>
+      <c r="E178" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F178">
+        <f t="shared" si="5"/>
+        <v>230</v>
+      </c>
+      <c r="G178" s="22" t="s">
+        <v>93</v>
+      </c>
       <c r="I178">
         <v>0</v>
       </c>
     </row>
-    <row r="179" spans="9:9">
+    <row r="179" spans="1:9" ht="25">
+      <c r="A179" s="1">
+        <v>42053</v>
+      </c>
+      <c r="B179">
+        <v>226.9</v>
+      </c>
+      <c r="C179" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="D179" s="20">
+        <v>8</v>
+      </c>
+      <c r="E179" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F179">
+        <f t="shared" si="5"/>
+        <v>230</v>
+      </c>
+      <c r="G179" s="22" t="s">
+        <v>93</v>
+      </c>
       <c r="I179">
         <v>0</v>
       </c>
     </row>
-    <row r="180" spans="9:9">
+    <row r="180" spans="1:9" ht="25">
+      <c r="A180" s="1">
+        <v>42053</v>
+      </c>
+      <c r="B180">
+        <v>226.9</v>
+      </c>
+      <c r="C180" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="D180" s="20">
+        <v>8</v>
+      </c>
+      <c r="E180" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F180">
+        <f t="shared" si="5"/>
+        <v>230</v>
+      </c>
+      <c r="G180" s="22" t="s">
+        <v>93</v>
+      </c>
       <c r="I180">
         <v>0</v>
       </c>
     </row>
-    <row r="181" spans="9:9">
+    <row r="181" spans="1:9" ht="25">
+      <c r="A181" s="1">
+        <v>42054</v>
+      </c>
+      <c r="B181">
+        <v>176.1</v>
+      </c>
+      <c r="C181" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D181" s="20">
+        <v>0</v>
+      </c>
+      <c r="E181" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F181">
+        <f t="shared" si="5"/>
+        <v>180</v>
+      </c>
+      <c r="G181" s="22" t="s">
+        <v>94</v>
+      </c>
       <c r="I181">
         <v>0</v>
       </c>
     </row>
-    <row r="182" spans="9:9">
+    <row r="182" spans="1:9" ht="25">
+      <c r="A182" s="1">
+        <v>42054</v>
+      </c>
+      <c r="B182">
+        <v>219.4</v>
+      </c>
+      <c r="C182" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D182" s="20">
+        <v>8</v>
+      </c>
+      <c r="E182" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F182">
+        <f t="shared" si="5"/>
+        <v>220</v>
+      </c>
+      <c r="G182" s="22" t="s">
+        <v>95</v>
+      </c>
       <c r="I182">
         <v>0</v>
       </c>
     </row>
-    <row r="183" spans="9:9">
+    <row r="183" spans="1:9" ht="25">
+      <c r="A183" s="1">
+        <v>42054</v>
+      </c>
+      <c r="B183">
+        <v>197.2</v>
+      </c>
+      <c r="C183" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="D183" s="20">
+        <v>8</v>
+      </c>
+      <c r="E183" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F183">
+        <f t="shared" si="5"/>
+        <v>200</v>
+      </c>
+      <c r="G183" s="22" t="s">
+        <v>96</v>
+      </c>
       <c r="I183">
         <v>0</v>
       </c>
     </row>
-    <row r="184" spans="9:9">
+    <row r="184" spans="1:9" ht="25">
+      <c r="A184" s="1">
+        <v>42054</v>
+      </c>
+      <c r="B184">
+        <v>221</v>
+      </c>
+      <c r="C184" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="D184" s="20">
+        <v>8</v>
+      </c>
+      <c r="E184" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F184">
+        <f t="shared" si="5"/>
+        <v>220</v>
+      </c>
+      <c r="G184" s="22" t="s">
+        <v>97</v>
+      </c>
       <c r="I184">
         <v>0</v>
       </c>
     </row>
-    <row r="185" spans="9:9">
+    <row r="185" spans="1:9" ht="25">
+      <c r="A185" s="1">
+        <v>42055</v>
+      </c>
+      <c r="B185">
+        <v>211.3</v>
+      </c>
+      <c r="C185" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D185" s="20">
+        <v>0</v>
+      </c>
+      <c r="E185" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F185">
+        <f t="shared" si="5"/>
+        <v>210</v>
+      </c>
+      <c r="G185" s="22" t="s">
+        <v>98</v>
+      </c>
       <c r="I185">
         <v>0</v>
       </c>
     </row>
-    <row r="186" spans="9:9">
+    <row r="186" spans="1:9" ht="25">
+      <c r="A186" s="1">
+        <v>42055</v>
+      </c>
+      <c r="B186">
+        <v>269</v>
+      </c>
+      <c r="C186" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D186" s="20">
+        <v>8</v>
+      </c>
+      <c r="E186" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F186">
+        <f t="shared" si="5"/>
+        <v>270</v>
+      </c>
+      <c r="G186" s="22" t="s">
+        <v>99</v>
+      </c>
       <c r="I186">
         <v>0</v>
       </c>
     </row>
-    <row r="187" spans="9:9">
+    <row r="187" spans="1:9" ht="25">
+      <c r="A187" s="1">
+        <v>42055</v>
+      </c>
+      <c r="B187">
+        <v>228</v>
+      </c>
+      <c r="C187" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="D187" s="20">
+        <v>8</v>
+      </c>
+      <c r="E187" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F187">
+        <f t="shared" si="5"/>
+        <v>230</v>
+      </c>
+      <c r="G187" s="22" t="s">
+        <v>100</v>
+      </c>
       <c r="I187">
         <v>0</v>
       </c>
     </row>
-    <row r="188" spans="9:9">
+    <row r="188" spans="1:9" ht="25">
+      <c r="A188" s="1">
+        <v>42055</v>
+      </c>
+      <c r="B188">
+        <v>250.8</v>
+      </c>
+      <c r="C188" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="D188" s="20">
+        <v>8</v>
+      </c>
+      <c r="E188" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F188">
+        <f t="shared" si="5"/>
+        <v>250</v>
+      </c>
+      <c r="G188" s="22" t="s">
+        <v>101</v>
+      </c>
       <c r="I188">
         <v>0</v>
       </c>
     </row>
-    <row r="189" spans="9:9">
+    <row r="189" spans="1:9" ht="25">
+      <c r="A189" s="1">
+        <v>42055</v>
+      </c>
+      <c r="B189">
+        <v>168.3</v>
+      </c>
+      <c r="C189" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D189" s="20">
+        <v>0</v>
+      </c>
+      <c r="E189" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F189">
+        <f t="shared" si="5"/>
+        <v>170</v>
+      </c>
+      <c r="G189" s="22" t="s">
+        <v>102</v>
+      </c>
       <c r="I189">
         <v>0</v>
       </c>
     </row>
-    <row r="190" spans="9:9">
+    <row r="190" spans="1:9" ht="25">
+      <c r="A190" s="1">
+        <v>42055</v>
+      </c>
+      <c r="B190">
+        <v>152.80000000000001</v>
+      </c>
+      <c r="C190" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D190" s="20">
+        <v>8</v>
+      </c>
+      <c r="E190" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F190">
+        <f t="shared" si="5"/>
+        <v>150</v>
+      </c>
+      <c r="G190" s="22" t="s">
+        <v>103</v>
+      </c>
       <c r="I190">
         <v>0</v>
       </c>
     </row>
-    <row r="191" spans="9:9">
+    <row r="191" spans="1:9" ht="25">
+      <c r="A191" s="1">
+        <v>42055</v>
+      </c>
+      <c r="B191">
+        <v>158.1</v>
+      </c>
+      <c r="C191" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="D191" s="20">
+        <v>8</v>
+      </c>
+      <c r="E191" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F191">
+        <f t="shared" si="5"/>
+        <v>160</v>
+      </c>
+      <c r="G191" s="22" t="s">
+        <v>104</v>
+      </c>
       <c r="I191">
         <v>0</v>
       </c>
     </row>
-    <row r="192" spans="9:9">
+    <row r="192" spans="1:9" ht="25">
+      <c r="A192" s="1">
+        <v>42055</v>
+      </c>
+      <c r="B192">
+        <v>175.8</v>
+      </c>
+      <c r="C192" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="D192" s="20">
+        <v>8</v>
+      </c>
+      <c r="E192" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F192">
+        <f t="shared" si="5"/>
+        <v>180</v>
+      </c>
+      <c r="G192" s="22" t="s">
+        <v>105</v>
+      </c>
       <c r="I192">
         <v>0</v>
       </c>
     </row>
-    <row r="193" spans="9:9">
+    <row r="193" spans="1:9" ht="25">
+      <c r="A193" s="1">
+        <v>42056</v>
+      </c>
+      <c r="B193">
+        <v>216.5</v>
+      </c>
+      <c r="C193" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D193" s="20">
+        <v>0</v>
+      </c>
+      <c r="E193" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F193">
+        <f t="shared" si="5"/>
+        <v>220</v>
+      </c>
+      <c r="G193" s="22" t="s">
+        <v>106</v>
+      </c>
       <c r="I193">
         <v>0</v>
       </c>
     </row>
-    <row r="194" spans="9:9">
+    <row r="194" spans="1:9" ht="25">
+      <c r="A194" s="1">
+        <v>42056</v>
+      </c>
+      <c r="B194">
+        <v>216.5</v>
+      </c>
+      <c r="C194" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D194" s="20">
+        <v>8</v>
+      </c>
+      <c r="E194" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F194">
+        <f t="shared" si="5"/>
+        <v>220</v>
+      </c>
+      <c r="G194" s="22" t="s">
+        <v>106</v>
+      </c>
       <c r="I194">
         <v>0</v>
       </c>
     </row>
-    <row r="195" spans="9:9">
+    <row r="195" spans="1:9" ht="25">
+      <c r="A195" s="1">
+        <v>42056</v>
+      </c>
+      <c r="B195">
+        <v>238.3</v>
+      </c>
+      <c r="C195" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="D195" s="20">
+        <v>8</v>
+      </c>
+      <c r="E195" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F195">
+        <f t="shared" si="5"/>
+        <v>240</v>
+      </c>
+      <c r="G195" s="22" t="s">
+        <v>107</v>
+      </c>
       <c r="I195">
         <v>0</v>
       </c>
     </row>
-    <row r="196" spans="9:9">
+    <row r="196" spans="1:9" ht="25">
+      <c r="A196" s="1">
+        <v>42056</v>
+      </c>
+      <c r="B196">
+        <v>256.7</v>
+      </c>
+      <c r="C196" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="D196" s="20">
+        <v>8</v>
+      </c>
+      <c r="E196" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F196">
+        <f t="shared" si="5"/>
+        <v>260</v>
+      </c>
+      <c r="G196" s="22" t="s">
+        <v>108</v>
+      </c>
       <c r="I196">
         <v>0</v>
       </c>
     </row>
-    <row r="197" spans="9:9">
+    <row r="197" spans="1:9" ht="25">
+      <c r="A197" s="1">
+        <v>42056</v>
+      </c>
+      <c r="B197">
+        <v>231.9</v>
+      </c>
+      <c r="C197" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D197" s="20">
+        <v>0</v>
+      </c>
+      <c r="E197" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F197">
+        <f t="shared" si="5"/>
+        <v>230</v>
+      </c>
+      <c r="G197" s="22" t="s">
+        <v>109</v>
+      </c>
       <c r="I197">
         <v>0</v>
       </c>
     </row>
-    <row r="198" spans="9:9">
+    <row r="198" spans="1:9" ht="25">
+      <c r="A198" s="1">
+        <v>42056</v>
+      </c>
+      <c r="B198">
+        <v>231.9</v>
+      </c>
+      <c r="C198" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D198" s="20">
+        <v>8</v>
+      </c>
+      <c r="E198" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F198">
+        <f t="shared" si="5"/>
+        <v>230</v>
+      </c>
+      <c r="G198" s="22" t="s">
+        <v>109</v>
+      </c>
       <c r="I198">
         <v>0</v>
       </c>
     </row>
-    <row r="199" spans="9:9">
+    <row r="199" spans="1:9" ht="25">
+      <c r="A199" s="1">
+        <v>42056</v>
+      </c>
+      <c r="B199">
+        <v>208.9</v>
+      </c>
+      <c r="C199" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="D199" s="20">
+        <v>8</v>
+      </c>
+      <c r="E199" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F199">
+        <f t="shared" si="5"/>
+        <v>210</v>
+      </c>
+      <c r="G199" s="22" t="s">
+        <v>110</v>
+      </c>
       <c r="I199">
         <v>0</v>
       </c>
     </row>
-    <row r="200" spans="9:9">
+    <row r="200" spans="1:9" ht="25">
+      <c r="A200" s="1">
+        <v>42056</v>
+      </c>
+      <c r="B200">
+        <v>231.9</v>
+      </c>
+      <c r="C200" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="D200" s="20">
+        <v>8</v>
+      </c>
+      <c r="E200" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F200">
+        <f t="shared" si="5"/>
+        <v>230</v>
+      </c>
+      <c r="G200" s="22" t="s">
+        <v>109</v>
+      </c>
       <c r="I200">
         <v>0</v>
       </c>
     </row>
+    <row r="201" spans="1:9" ht="25">
+      <c r="A201" s="1">
+        <v>42057</v>
+      </c>
+      <c r="B201">
+        <v>207.9</v>
+      </c>
+      <c r="C201" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D201" s="20">
+        <v>0</v>
+      </c>
+      <c r="E201" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F201">
+        <f t="shared" si="5"/>
+        <v>210</v>
+      </c>
+      <c r="G201" s="22" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="202" spans="1:9" ht="25">
+      <c r="A202" s="1">
+        <v>42057</v>
+      </c>
+      <c r="B202">
+        <v>188.7</v>
+      </c>
+      <c r="C202" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D202" s="20">
+        <v>8</v>
+      </c>
+      <c r="E202" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F202">
+        <f t="shared" si="5"/>
+        <v>190</v>
+      </c>
+      <c r="G202" s="22" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="203" spans="1:9" ht="25">
+      <c r="A203" s="1">
+        <v>42057</v>
+      </c>
+      <c r="B203">
+        <v>205.3</v>
+      </c>
+      <c r="C203" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="D203" s="20">
+        <v>8</v>
+      </c>
+      <c r="E203" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F203">
+        <f t="shared" si="5"/>
+        <v>210</v>
+      </c>
+      <c r="G203" s="22" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="204" spans="1:9" ht="25">
+      <c r="A204" s="1">
+        <v>42057</v>
+      </c>
+      <c r="B204">
+        <v>189</v>
+      </c>
+      <c r="C204" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="D204" s="20">
+        <v>8</v>
+      </c>
+      <c r="E204" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F204">
+        <f t="shared" si="5"/>
+        <v>190</v>
+      </c>
+      <c r="G204" s="22" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="205" spans="1:9" ht="25">
+      <c r="A205" s="1">
+        <v>42058</v>
+      </c>
+      <c r="B205">
+        <v>200.7</v>
+      </c>
+      <c r="C205" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D205" s="20">
+        <v>0</v>
+      </c>
+      <c r="E205" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F205">
+        <f t="shared" si="5"/>
+        <v>200</v>
+      </c>
+      <c r="G205" s="22" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="206" spans="1:9" ht="25">
+      <c r="A206" s="1">
+        <v>42058</v>
+      </c>
+      <c r="B206">
+        <v>200.7</v>
+      </c>
+      <c r="C206" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D206" s="20">
+        <v>8</v>
+      </c>
+      <c r="E206" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F206">
+        <f t="shared" si="5"/>
+        <v>200</v>
+      </c>
+      <c r="G206" s="22" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="207" spans="1:9" ht="25">
+      <c r="A207" s="1">
+        <v>42058</v>
+      </c>
+      <c r="B207">
+        <v>158.1</v>
+      </c>
+      <c r="C207" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="D207" s="20">
+        <v>8</v>
+      </c>
+      <c r="E207" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F207">
+        <f t="shared" si="5"/>
+        <v>160</v>
+      </c>
+      <c r="G207" s="22" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="208" spans="1:9" ht="25">
+      <c r="A208" s="1">
+        <v>42058</v>
+      </c>
+      <c r="B208">
+        <v>212.7</v>
+      </c>
+      <c r="C208" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="D208" s="20">
+        <v>8</v>
+      </c>
+      <c r="E208" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F208">
+        <f t="shared" si="5"/>
+        <v>210</v>
+      </c>
+      <c r="G208" s="22" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="209" spans="1:7" ht="25">
+      <c r="A209" s="1">
+        <v>42059</v>
+      </c>
+      <c r="B209">
+        <v>218.3</v>
+      </c>
+      <c r="C209" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D209" s="20">
+        <v>0</v>
+      </c>
+      <c r="E209" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F209">
+        <f t="shared" si="5"/>
+        <v>220</v>
+      </c>
+      <c r="G209" s="22" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="210" spans="1:7" ht="25">
+      <c r="A210" s="1">
+        <v>42059</v>
+      </c>
+      <c r="B210">
+        <v>231.9</v>
+      </c>
+      <c r="C210" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D210" s="20">
+        <v>8</v>
+      </c>
+      <c r="E210" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F210">
+        <f t="shared" si="5"/>
+        <v>230</v>
+      </c>
+      <c r="G210" s="22" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="211" spans="1:7" ht="25">
+      <c r="A211" s="1">
+        <v>42059</v>
+      </c>
+      <c r="B211">
+        <v>246.3</v>
+      </c>
+      <c r="C211" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="D211" s="20">
+        <v>8</v>
+      </c>
+      <c r="E211" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F211">
+        <f t="shared" si="5"/>
+        <v>250</v>
+      </c>
+      <c r="G211" s="22" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="212" spans="1:7" ht="25">
+      <c r="A212" s="1">
+        <v>42059</v>
+      </c>
+      <c r="B212">
+        <v>218.5</v>
+      </c>
+      <c r="C212" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="D212" s="20">
+        <v>8</v>
+      </c>
+      <c r="E212" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F212">
+        <f t="shared" si="5"/>
+        <v>220</v>
+      </c>
+      <c r="G212" s="22" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="213" spans="1:7" ht="25">
+      <c r="A213" s="1">
+        <v>42060</v>
+      </c>
+      <c r="B213">
+        <v>221</v>
+      </c>
+      <c r="C213" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D213" s="20">
+        <v>0</v>
+      </c>
+      <c r="E213" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F213">
+        <f t="shared" si="5"/>
+        <v>220</v>
+      </c>
+      <c r="G213" s="22" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="214" spans="1:7" ht="25">
+      <c r="A214" s="1">
+        <v>42060</v>
+      </c>
+      <c r="B214">
+        <v>188</v>
+      </c>
+      <c r="C214" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D214" s="20">
+        <v>8</v>
+      </c>
+      <c r="E214" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F214">
+        <f t="shared" si="5"/>
+        <v>190</v>
+      </c>
+      <c r="G214" s="22" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="215" spans="1:7" ht="25">
+      <c r="A215" s="1">
+        <v>42060</v>
+      </c>
+      <c r="B215">
+        <v>209.1</v>
+      </c>
+      <c r="C215" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="D215" s="20">
+        <v>8</v>
+      </c>
+      <c r="E215" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F215">
+        <f t="shared" si="5"/>
+        <v>210</v>
+      </c>
+      <c r="G215" s="22" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="216" spans="1:7" ht="25">
+      <c r="A216" s="1">
+        <v>42060</v>
+      </c>
+      <c r="B216">
+        <v>192</v>
+      </c>
+      <c r="C216" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="D216" s="20">
+        <v>8</v>
+      </c>
+      <c r="E216" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F216">
+        <f t="shared" si="5"/>
+        <v>190</v>
+      </c>
+      <c r="G216" s="22" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="217" spans="1:7" ht="25">
+      <c r="A217" s="1">
+        <v>42062</v>
+      </c>
+      <c r="B217">
+        <v>171.4</v>
+      </c>
+      <c r="C217" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D217" s="20">
+        <v>0</v>
+      </c>
+      <c r="E217" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F217">
+        <f t="shared" si="5"/>
+        <v>170</v>
+      </c>
+      <c r="G217" s="22" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="218" spans="1:7" ht="25">
+      <c r="A218" s="1">
+        <v>42062</v>
+      </c>
+      <c r="B218">
+        <v>171.4</v>
+      </c>
+      <c r="C218" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D218" s="20">
+        <v>8</v>
+      </c>
+      <c r="E218" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F218">
+        <f t="shared" si="5"/>
+        <v>170</v>
+      </c>
+      <c r="G218" s="22" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="219" spans="1:7" ht="25">
+      <c r="A219" s="1">
+        <v>42062</v>
+      </c>
+      <c r="B219">
+        <v>174.2</v>
+      </c>
+      <c r="C219" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="D219" s="20">
+        <v>8</v>
+      </c>
+      <c r="E219" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F219">
+        <f t="shared" si="5"/>
+        <v>170</v>
+      </c>
+      <c r="G219" s="22" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="220" spans="1:7" ht="25">
+      <c r="A220" s="1">
+        <v>42062</v>
+      </c>
+      <c r="B220">
+        <v>184.7</v>
+      </c>
+      <c r="C220" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="D220" s="20">
+        <v>8</v>
+      </c>
+      <c r="E220" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F220">
+        <f t="shared" si="5"/>
+        <v>180</v>
+      </c>
+      <c r="G220" s="22" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="221" spans="1:7" ht="25">
+      <c r="A221" s="1">
+        <v>42063</v>
+      </c>
+      <c r="B221">
+        <v>228.1</v>
+      </c>
+      <c r="C221" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D221" s="20">
+        <v>0</v>
+      </c>
+      <c r="E221" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F221">
+        <f t="shared" si="5"/>
+        <v>230</v>
+      </c>
+      <c r="G221" s="22" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="222" spans="1:7" ht="25">
+      <c r="A222" s="1">
+        <v>42063</v>
+      </c>
+      <c r="B222">
+        <v>206.5</v>
+      </c>
+      <c r="C222" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D222" s="20">
+        <v>8</v>
+      </c>
+      <c r="E222" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F222">
+        <f t="shared" si="5"/>
+        <v>210</v>
+      </c>
+      <c r="G222" s="22" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="223" spans="1:7" ht="25">
+      <c r="A223" s="1">
+        <v>42063</v>
+      </c>
+      <c r="B223">
+        <v>221.9</v>
+      </c>
+      <c r="C223" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="D223" s="20">
+        <v>8</v>
+      </c>
+      <c r="E223" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F223">
+        <f t="shared" si="5"/>
+        <v>220</v>
+      </c>
+      <c r="G223" s="22" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="224" spans="1:7" ht="25">
+      <c r="A224" s="1">
+        <v>42063</v>
+      </c>
+      <c r="B224">
+        <v>221.9</v>
+      </c>
+      <c r="C224" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="D224" s="20">
+        <v>8</v>
+      </c>
+      <c r="E224" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F224">
+        <f t="shared" si="5"/>
+        <v>220</v>
+      </c>
+      <c r="G224" s="22" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="225" spans="1:7" ht="25">
+      <c r="A225" s="1">
+        <v>42064</v>
+      </c>
+      <c r="B225">
+        <v>235.7</v>
+      </c>
+      <c r="C225" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D225" s="20">
+        <v>0</v>
+      </c>
+      <c r="E225" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F225">
+        <f t="shared" si="5"/>
+        <v>240</v>
+      </c>
+      <c r="G225" s="22" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="226" spans="1:7" ht="25">
+      <c r="A226" s="1">
+        <v>42064</v>
+      </c>
+      <c r="B226">
+        <v>205.8</v>
+      </c>
+      <c r="C226" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D226" s="20">
+        <v>8</v>
+      </c>
+      <c r="E226" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F226">
+        <f t="shared" si="5"/>
+        <v>210</v>
+      </c>
+      <c r="G226" s="22" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="227" spans="1:7" ht="25">
+      <c r="A227" s="1">
+        <v>42064</v>
+      </c>
+      <c r="B227">
+        <v>257.2</v>
+      </c>
+      <c r="C227" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="D227" s="20">
+        <v>8</v>
+      </c>
+      <c r="E227" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F227">
+        <f t="shared" si="5"/>
+        <v>260</v>
+      </c>
+      <c r="G227" s="22" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="228" spans="1:7" ht="25">
+      <c r="A228" s="1">
+        <v>42064</v>
+      </c>
+      <c r="B228">
+        <v>206</v>
+      </c>
+      <c r="C228" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="D228" s="20">
+        <v>8</v>
+      </c>
+      <c r="E228" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F228">
+        <f t="shared" si="5"/>
+        <v>210</v>
+      </c>
+      <c r="G228" s="22" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="229" spans="1:7" ht="25">
+      <c r="A229" s="1">
+        <v>42064</v>
+      </c>
+      <c r="B229">
+        <v>202.2</v>
+      </c>
+      <c r="C229" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D229" s="20">
+        <v>0</v>
+      </c>
+      <c r="E229" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F229">
+        <f t="shared" si="5"/>
+        <v>200</v>
+      </c>
+      <c r="G229" s="22" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="230" spans="1:7" ht="25">
+      <c r="A230" s="1">
+        <v>42064</v>
+      </c>
+      <c r="B230">
+        <v>202.2</v>
+      </c>
+      <c r="C230" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D230" s="20">
+        <v>8</v>
+      </c>
+      <c r="E230" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F230">
+        <f t="shared" si="5"/>
+        <v>200</v>
+      </c>
+      <c r="G230" s="22" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="231" spans="1:7" ht="25">
+      <c r="A231" s="1">
+        <v>42064</v>
+      </c>
+      <c r="B231">
+        <v>185.9</v>
+      </c>
+      <c r="C231" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="D231" s="20">
+        <v>8</v>
+      </c>
+      <c r="E231" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F231">
+        <f t="shared" si="5"/>
+        <v>190</v>
+      </c>
+      <c r="G231" s="22" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="232" spans="1:7" ht="25">
+      <c r="A232" s="1">
+        <v>42064</v>
+      </c>
+      <c r="B232">
+        <v>202.2</v>
+      </c>
+      <c r="C232" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="D232" s="20">
+        <v>8</v>
+      </c>
+      <c r="E232" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F232">
+        <f t="shared" si="5"/>
+        <v>200</v>
+      </c>
+      <c r="G232" s="22" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="233" spans="1:7" ht="25">
+      <c r="A233" s="23">
+        <v>42065</v>
+      </c>
+      <c r="B233">
+        <v>202.1</v>
+      </c>
+      <c r="C233" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D233" s="20">
+        <v>0</v>
+      </c>
+      <c r="E233" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F233">
+        <f t="shared" si="5"/>
+        <v>200</v>
+      </c>
+      <c r="G233" s="22" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="234" spans="1:7" ht="25">
+      <c r="A234" s="1">
+        <v>42065</v>
+      </c>
+      <c r="B234">
+        <v>202.1</v>
+      </c>
+      <c r="C234" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D234" s="20">
+        <v>8</v>
+      </c>
+      <c r="E234" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F234">
+        <f t="shared" ref="F234:F236" si="6">ROUND(B234/10,0)*10</f>
+        <v>200</v>
+      </c>
+      <c r="G234" s="22" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="235" spans="1:7" ht="25">
+      <c r="A235" s="1">
+        <v>42065</v>
+      </c>
+      <c r="B235">
+        <v>197.4</v>
+      </c>
+      <c r="C235" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="D235" s="20">
+        <v>8</v>
+      </c>
+      <c r="E235" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F235">
+        <f t="shared" si="6"/>
+        <v>200</v>
+      </c>
+      <c r="G235" s="22" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="236" spans="1:7" ht="25">
+      <c r="A236" s="1">
+        <v>42065</v>
+      </c>
+      <c r="B236">
+        <v>202.1</v>
+      </c>
+      <c r="C236" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="D236" s="20">
+        <v>8</v>
+      </c>
+      <c r="E236" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F236">
+        <f t="shared" si="6"/>
+        <v>200</v>
+      </c>
+      <c r="G236" s="22" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="237" spans="1:7" ht="25">
+      <c r="A237" s="1">
+        <v>42066</v>
+      </c>
+      <c r="C237" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D237" s="20">
+        <v>0</v>
+      </c>
+      <c r="E237" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="G237" s="22" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="238" spans="1:7" ht="25">
+      <c r="A238" s="1">
+        <v>42066</v>
+      </c>
+      <c r="C238" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D238" s="20">
+        <v>8</v>
+      </c>
+      <c r="E238" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="G238" s="22" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="239" spans="1:7" ht="25">
+      <c r="A239" s="1">
+        <v>42066</v>
+      </c>
+      <c r="C239" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="D239" s="20">
+        <v>8</v>
+      </c>
+      <c r="E239" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="G239" s="22" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="240" spans="1:7" ht="25">
+      <c r="A240" s="1">
+        <v>42066</v>
+      </c>
+      <c r="C240" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="D240" s="20">
+        <v>8</v>
+      </c>
+      <c r="E240" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="G240" s="22" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="241" spans="1:7" ht="25">
+      <c r="A241" s="1">
+        <v>42067</v>
+      </c>
+      <c r="C241" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D241" s="20">
+        <v>0</v>
+      </c>
+      <c r="E241" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="G241" s="22" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="242" spans="1:7" ht="25">
+      <c r="A242" s="1">
+        <v>42067</v>
+      </c>
+      <c r="C242" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D242" s="20">
+        <v>8</v>
+      </c>
+      <c r="E242" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="G242" s="22" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="243" spans="1:7" ht="25">
+      <c r="A243" s="1">
+        <v>42067</v>
+      </c>
+      <c r="C243" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="D243" s="20">
+        <v>8</v>
+      </c>
+      <c r="E243" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="G243" s="22" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="244" spans="1:7" ht="25">
+      <c r="A244" s="1">
+        <v>42067</v>
+      </c>
+      <c r="C244" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="D244" s="20">
+        <v>8</v>
+      </c>
+      <c r="E244" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="G244" s="22" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="1048576" spans="1:1">
+      <c r="A1048576" s="1"/>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="G212" r:id="rId1"/>
+    <hyperlink ref="G223" r:id="rId2"/>
+    <hyperlink ref="G224" r:id="rId3"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967292" verticalDpi="4294967292"/>
   <extLst>

</xml_diff>